<commit_message>
updated calendar and initial push for tuotring
</commit_message>
<xml_diff>
--- a/CS320-Spring2025Calendar.xlsx
+++ b/CS320-Spring2025Calendar.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="28227"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="28324"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\cygwin64\home\donha\cs320-spring2025\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{473C1589-7FBC-4E6B-8BAD-674C5E2BC6B7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{32F16F28-CA49-4963-AD2D-27275D190D10}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2730" yWindow="1935" windowWidth="18180" windowHeight="14265" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="14940" yWindow="915" windowWidth="13665" windowHeight="14265" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Calendar-Sp24" sheetId="1" r:id="rId1"/>
@@ -232,12 +232,6 @@
 Web Applications Labs Review</t>
   </si>
   <si>
-    <t>A01: Team Project Proposal due 7:00a, 
-Wed, 2-14-24
----------&gt;&gt;&gt;&gt;
-(Marmoset)</t>
-  </si>
-  <si>
     <t>A05: Team Final Use Cases
 due Noon
 (Google Doc)
@@ -318,10 +312,6 @@
     <t>A08: Team Project Report
  due Noon
 (Marmoset)</t>
-  </si>
-  <si>
-    <t>CS320: SW Engineering - Spring 2025 Schedule
-(as of 1-6-2025, subject to change)</t>
   </si>
   <si>
     <t xml:space="preserve">Reading Day
@@ -490,21 +480,6 @@
 (Marmoset)</t>
   </si>
   <si>
-    <t xml:space="preserve">Lab 2a: Web Apps Lab02a due
-Mon before class
--------------&gt;&gt;&gt;&gt;
- (after sign-off)
-(Marmoset)
-</t>
-  </si>
-  <si>
-    <t xml:space="preserve">
-A09: Individual  Report 
-due Weds before class
------&gt;&gt;&gt;&gt;&gt;
-(Marmoset)</t>
-  </si>
-  <si>
     <t>Lab 5: JDBC
 due Mon before class
 -------------&gt;&gt;&gt;&gt;
@@ -532,6 +507,28 @@
       </rPr>
       <t>A06: Problem Domain (assigned)</t>
     </r>
+  </si>
+  <si>
+    <t>A01: Team Project Proposal due Noon
+(Marmoset)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Lab 2a: Web Apps Lab02a due
+Noon
+(after sign-off)
+(Marmoset)
+</t>
+  </si>
+  <si>
+    <t>CS320: SW Engineering - Spring 2025 Schedule
+(as of 1-25-2025, subject to change)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">
+A09: Individual  Report 
+due Weds by Noon
+-----&gt;&gt;&gt;&gt;&gt;
+(Marmoset)</t>
   </si>
 </sst>
 </file>
@@ -1194,7 +1191,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="159">
+  <cellXfs count="161">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -1295,9 +1292,6 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1418,9 +1412,6 @@
     <xf numFmtId="0" fontId="7" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="6" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1442,9 +1433,6 @@
     <xf numFmtId="0" fontId="5" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1455,9 +1443,6 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="6" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="2" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1589,9 +1574,6 @@
     <xf numFmtId="0" fontId="5" fillId="3" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1612,6 +1594,30 @@
     </xf>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
@@ -1622,39 +1628,21 @@
     <xf numFmtId="0" fontId="2" fillId="2" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1664,11 +1652,26 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1997,17 +2000,17 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:17" ht="53.1" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="145" t="s">
-        <v>55</v>
-      </c>
-      <c r="B1" s="146"/>
-      <c r="C1" s="146"/>
-      <c r="D1" s="146"/>
-      <c r="E1" s="146"/>
-      <c r="F1" s="146"/>
-      <c r="G1" s="146"/>
-      <c r="H1" s="146"/>
-      <c r="I1" s="147"/>
+      <c r="A1" s="146" t="s">
+        <v>79</v>
+      </c>
+      <c r="B1" s="147"/>
+      <c r="C1" s="147"/>
+      <c r="D1" s="147"/>
+      <c r="E1" s="147"/>
+      <c r="F1" s="147"/>
+      <c r="G1" s="147"/>
+      <c r="H1" s="147"/>
+      <c r="I1" s="148"/>
     </row>
     <row r="2" spans="1:17" s="2" customFormat="1" ht="21" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
@@ -2029,7 +2032,7 @@
       <c r="G2" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="H2" s="101" t="s">
+      <c r="H2" s="97" t="s">
         <v>4</v>
       </c>
       <c r="I2" s="1" t="s">
@@ -2037,20 +2040,20 @@
       </c>
     </row>
     <row r="3" spans="1:17" ht="15.75" customHeight="1" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="149">
+      <c r="A3" s="137">
         <v>15</v>
       </c>
-      <c r="B3" s="140" t="s">
-        <v>60</v>
-      </c>
-      <c r="C3" s="53">
+      <c r="B3" s="143" t="s">
+        <v>58</v>
+      </c>
+      <c r="C3" s="52">
         <v>26</v>
       </c>
-      <c r="D3" s="43">
+      <c r="D3" s="42">
         <f>C3 + 1</f>
         <v>27</v>
       </c>
-      <c r="E3" s="43">
+      <c r="E3" s="42">
         <f t="shared" ref="E3:H3" si="0">D3 + 1</f>
         <v>28</v>
       </c>
@@ -2062,45 +2065,45 @@
         <f t="shared" si="0"/>
         <v>30</v>
       </c>
-      <c r="H3" s="102">
+      <c r="H3" s="98">
         <f t="shared" si="0"/>
         <v>31</v>
       </c>
-      <c r="I3" s="103">
+      <c r="I3" s="99">
         <f>IF(H3 = 31, 1, H3+1)</f>
         <v>1</v>
       </c>
     </row>
     <row r="4" spans="1:17" ht="147" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="150"/>
-      <c r="B4" s="142"/>
-      <c r="C4" s="104" t="s">
+      <c r="A4" s="138"/>
+      <c r="B4" s="145"/>
+      <c r="C4" s="100" t="s">
         <v>7</v>
       </c>
-      <c r="D4" s="99" t="s">
+      <c r="D4" s="95" t="s">
+        <v>59</v>
+      </c>
+      <c r="E4" s="86" t="s">
+        <v>72</v>
+      </c>
+      <c r="F4" s="123" t="s">
         <v>61</v>
       </c>
-      <c r="E4" s="90" t="s">
-        <v>74</v>
-      </c>
-      <c r="F4" s="127" t="s">
-        <v>63</v>
-      </c>
       <c r="G4" s="32"/>
-      <c r="H4" s="128" t="s">
+      <c r="H4" s="124" t="s">
         <v>37</v>
       </c>
-      <c r="I4" s="106"/>
+      <c r="I4" s="102"/>
     </row>
     <row r="5" spans="1:17" ht="15" customHeight="1" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="151">
+      <c r="A5" s="149">
         <f>A3 - 1</f>
         <v>14</v>
       </c>
-      <c r="B5" s="143" t="s">
+      <c r="B5" s="150" t="s">
         <v>10</v>
       </c>
-      <c r="C5" s="105">
+      <c r="C5" s="101">
         <f>I3 + 1</f>
         <v>2</v>
       </c>
@@ -2130,30 +2133,30 @@
       </c>
     </row>
     <row r="6" spans="1:17" ht="90.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="152"/>
-      <c r="B6" s="144"/>
-      <c r="C6" s="129"/>
-      <c r="D6" s="39" t="s">
+      <c r="A6" s="136"/>
+      <c r="B6" s="141"/>
+      <c r="C6" s="125"/>
+      <c r="D6" s="38" t="s">
+        <v>71</v>
+      </c>
+      <c r="E6" s="39" t="s">
         <v>73</v>
       </c>
-      <c r="E6" s="40" t="s">
-        <v>75</v>
-      </c>
-      <c r="F6" s="39" t="s">
-        <v>64</v>
-      </c>
-      <c r="G6" s="62"/>
-      <c r="H6" s="39" t="s">
-        <v>65</v>
-      </c>
-      <c r="I6" s="72"/>
+      <c r="F6" s="38" t="s">
+        <v>62</v>
+      </c>
+      <c r="G6" s="61"/>
+      <c r="H6" s="38" t="s">
+        <v>63</v>
+      </c>
+      <c r="I6" s="71"/>
     </row>
     <row r="7" spans="1:17" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="153">
+      <c r="A7" s="135">
         <f>A5 - 1</f>
         <v>13</v>
       </c>
-      <c r="B7" s="144"/>
+      <c r="B7" s="141"/>
       <c r="C7" s="15">
         <f>I5 + 1</f>
         <v>9</v>
@@ -2178,36 +2181,36 @@
         <f>G7+1</f>
         <v>14</v>
       </c>
-      <c r="I7" s="41">
+      <c r="I7" s="40">
         <f>H7+1</f>
         <v>15</v>
       </c>
     </row>
     <row r="8" spans="1:17" ht="87" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="153"/>
-      <c r="B8" s="144"/>
-      <c r="C8" s="129"/>
+      <c r="A8" s="135"/>
+      <c r="B8" s="141"/>
+      <c r="C8" s="154" t="s">
+        <v>31</v>
+      </c>
       <c r="D8" s="11" t="s">
         <v>38</v>
       </c>
-      <c r="E8" s="83" t="s">
-        <v>31</v>
-      </c>
+      <c r="E8" s="155"/>
       <c r="F8" s="11" t="s">
         <v>40</v>
       </c>
       <c r="G8" s="24"/>
-      <c r="H8" s="137" t="s">
-        <v>66</v>
-      </c>
-      <c r="I8" s="84"/>
+      <c r="H8" s="132" t="s">
+        <v>64</v>
+      </c>
+      <c r="I8" s="81"/>
     </row>
     <row r="9" spans="1:17" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="153">
+      <c r="A9" s="135">
         <f>A7 - 1</f>
         <v>12</v>
       </c>
-      <c r="B9" s="144"/>
+      <c r="B9" s="141"/>
       <c r="C9" s="12">
         <f>I7 + 1</f>
         <v>16</v>
@@ -2236,47 +2239,49 @@
         <f t="shared" si="1"/>
         <v>22</v>
       </c>
-      <c r="K9" s="77"/>
-      <c r="L9" s="77"/>
-      <c r="M9" s="77"/>
-      <c r="N9" s="77"/>
-      <c r="O9" s="77"/>
-      <c r="P9" s="77"/>
-      <c r="Q9" s="77"/>
+      <c r="K9" s="75"/>
+      <c r="L9" s="75"/>
+      <c r="M9" s="75"/>
+      <c r="N9" s="75"/>
+      <c r="O9" s="75"/>
+      <c r="P9" s="75"/>
+      <c r="Q9" s="75"/>
     </row>
     <row r="10" spans="1:17" ht="102.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="153"/>
-      <c r="B10" s="144"/>
-      <c r="C10" s="73" t="s">
-        <v>41</v>
+      <c r="A10" s="135"/>
+      <c r="B10" s="141"/>
+      <c r="C10" s="72" t="s">
+        <v>77</v>
       </c>
       <c r="D10" s="9" t="s">
         <v>39</v>
       </c>
-      <c r="E10" s="62"/>
+      <c r="E10" s="61"/>
       <c r="F10" s="9" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="G10" s="10"/>
       <c r="H10" s="9" t="s">
         <v>27</v>
       </c>
-      <c r="I10" s="34"/>
+      <c r="I10" s="157" t="s">
+        <v>78</v>
+      </c>
       <c r="K10" s="22"/>
-      <c r="L10" s="77"/>
-      <c r="M10" s="78"/>
-      <c r="N10" s="77"/>
-      <c r="O10" s="78"/>
-      <c r="P10" s="77"/>
-      <c r="Q10" s="78"/>
+      <c r="L10" s="75"/>
+      <c r="M10" s="76"/>
+      <c r="N10" s="75"/>
+      <c r="O10" s="76"/>
+      <c r="P10" s="75"/>
+      <c r="Q10" s="76"/>
     </row>
     <row r="11" spans="1:17" ht="15" customHeight="1" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="153">
+      <c r="A11" s="135">
         <f>A9 -1</f>
         <v>11</v>
       </c>
-      <c r="B11" s="143" t="s">
-        <v>62</v>
+      <c r="B11" s="150" t="s">
+        <v>60</v>
       </c>
       <c r="C11" s="15">
         <f>I9 + 1</f>
@@ -2298,161 +2303,159 @@
         <f t="shared" si="1"/>
         <v>27</v>
       </c>
-      <c r="H11" s="107">
+      <c r="H11" s="103">
         <f t="shared" si="1"/>
         <v>28</v>
       </c>
-      <c r="I11" s="113">
+      <c r="I11" s="109">
         <f>IF(H11 = 28,1,H11+1)</f>
         <v>1</v>
       </c>
-      <c r="K11" s="77"/>
-      <c r="L11" s="77"/>
-      <c r="M11" s="77"/>
-      <c r="N11" s="77"/>
-      <c r="O11" s="77"/>
-      <c r="P11" s="77"/>
-      <c r="Q11" s="77"/>
+      <c r="K11" s="75"/>
+      <c r="L11" s="75"/>
+      <c r="M11" s="75"/>
+      <c r="N11" s="75"/>
+      <c r="O11" s="75"/>
+      <c r="P11" s="75"/>
+      <c r="Q11" s="75"/>
     </row>
     <row r="12" spans="1:17" ht="120" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="152"/>
-      <c r="B12" s="148"/>
-      <c r="C12" s="88" t="s">
-        <v>76</v>
-      </c>
-      <c r="D12" s="92" t="s">
-        <v>45</v>
-      </c>
-      <c r="E12" s="130"/>
-      <c r="F12" s="131" t="s">
+      <c r="A12" s="136"/>
+      <c r="B12" s="142"/>
+      <c r="C12" s="156"/>
+      <c r="D12" s="158" t="s">
         <v>44</v>
       </c>
-      <c r="G12" s="35"/>
-      <c r="H12" s="132" t="s">
+      <c r="E12" s="126"/>
+      <c r="F12" s="127" t="s">
+        <v>43</v>
+      </c>
+      <c r="G12" s="34"/>
+      <c r="H12" s="160" t="s">
         <v>21</v>
       </c>
-      <c r="I12" s="114"/>
+      <c r="I12" s="110"/>
       <c r="K12" s="22"/>
-      <c r="L12" s="77"/>
-      <c r="M12" s="77"/>
-      <c r="N12" s="77"/>
-      <c r="O12" s="78"/>
-      <c r="P12" s="77"/>
-      <c r="Q12" s="78"/>
+      <c r="L12" s="75"/>
+      <c r="M12" s="75"/>
+      <c r="N12" s="75"/>
+      <c r="O12" s="76"/>
+      <c r="P12" s="75"/>
+      <c r="Q12" s="76"/>
     </row>
     <row r="13" spans="1:17" ht="15" customHeight="1" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="110">
+      <c r="A13" s="106">
         <f xml:space="preserve"> A11 - 1</f>
         <v>10</v>
       </c>
-      <c r="B13" s="140" t="s">
+      <c r="B13" s="143" t="s">
         <v>11</v>
       </c>
-      <c r="C13" s="111">
+      <c r="C13" s="107">
         <f>IF(I11=28, 1, I11+1)</f>
         <v>2</v>
       </c>
-      <c r="D13" s="63">
+      <c r="D13" s="62">
         <f>C13 + 1</f>
         <v>3</v>
       </c>
-      <c r="E13" s="43">
+      <c r="E13" s="42">
         <f t="shared" ref="E13:F13" si="2">D13 + 1</f>
         <v>4</v>
       </c>
-      <c r="F13" s="43">
+      <c r="F13" s="42">
         <f t="shared" si="2"/>
         <v>5</v>
       </c>
-      <c r="G13" s="54">
+      <c r="G13" s="53">
         <f>IF(F13 = 28, 1, F13+1)</f>
         <v>6</v>
       </c>
-      <c r="H13" s="54">
+      <c r="H13" s="53">
         <f>IF(G13 = 28, 1, G13+1)</f>
         <v>7</v>
       </c>
-      <c r="I13" s="66">
+      <c r="I13" s="65">
         <f t="shared" si="1"/>
         <v>8</v>
       </c>
-      <c r="K13" s="77"/>
-      <c r="L13" s="77"/>
-      <c r="M13" s="77"/>
-      <c r="N13" s="77"/>
-      <c r="O13" s="77"/>
-      <c r="P13" s="77"/>
-      <c r="Q13" s="79"/>
+      <c r="K13" s="75"/>
+      <c r="L13" s="75"/>
+      <c r="M13" s="75"/>
+      <c r="N13" s="75"/>
+      <c r="O13" s="75"/>
+      <c r="P13" s="75"/>
+      <c r="Q13" s="77"/>
     </row>
     <row r="14" spans="1:17" ht="144.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="109"/>
-      <c r="B14" s="141"/>
-      <c r="C14" s="87" t="s">
-        <v>42</v>
-      </c>
-      <c r="D14" s="85" t="s">
-        <v>80</v>
-      </c>
-      <c r="E14" s="112"/>
+      <c r="A14" s="105"/>
+      <c r="B14" s="144"/>
+      <c r="C14" s="84" t="s">
+        <v>41</v>
+      </c>
+      <c r="D14" s="82" t="s">
+        <v>76</v>
+      </c>
+      <c r="E14" s="108"/>
       <c r="F14" s="6" t="s">
-        <v>68</v>
-      </c>
-      <c r="G14" s="52" t="s">
+        <v>66</v>
+      </c>
+      <c r="G14" s="51" t="s">
         <v>28</v>
       </c>
-      <c r="H14" s="71" t="s">
+      <c r="H14" s="70" t="s">
         <v>28</v>
       </c>
-      <c r="I14" s="64" t="s">
+      <c r="I14" s="63" t="s">
         <v>28</v>
       </c>
-      <c r="K14" s="79"/>
+      <c r="K14" s="77"/>
       <c r="L14" s="22"/>
-      <c r="M14" s="80"/>
-      <c r="N14" s="77"/>
-      <c r="O14" s="79"/>
-      <c r="P14" s="77"/>
-      <c r="Q14" s="79"/>
+      <c r="M14" s="78"/>
+      <c r="N14" s="75"/>
+      <c r="O14" s="77"/>
+      <c r="P14" s="75"/>
+      <c r="Q14" s="77"/>
     </row>
     <row r="15" spans="1:17" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="94">
+      <c r="A15" s="90">
         <f>A13 - 1</f>
         <v>9</v>
       </c>
-      <c r="B15" s="141"/>
-      <c r="C15" s="55">
+      <c r="B15" s="144"/>
+      <c r="C15" s="54">
         <f>I13 + 1</f>
         <v>9</v>
       </c>
-      <c r="D15" s="44">
+      <c r="D15" s="43">
         <f t="shared" ref="D15:I15" si="3">C15 + 1</f>
         <v>10</v>
       </c>
-      <c r="E15" s="85">
+      <c r="E15" s="82">
         <f t="shared" si="3"/>
         <v>11</v>
       </c>
-      <c r="F15" s="44">
+      <c r="F15" s="43">
         <f t="shared" si="3"/>
         <v>12</v>
       </c>
-      <c r="G15" s="108">
+      <c r="G15" s="104">
         <f t="shared" si="3"/>
         <v>13</v>
       </c>
-      <c r="H15" s="44">
+      <c r="H15" s="43">
         <f t="shared" si="3"/>
         <v>14</v>
       </c>
-      <c r="I15" s="67">
+      <c r="I15" s="66">
         <f t="shared" si="3"/>
         <v>15</v>
       </c>
     </row>
     <row r="16" spans="1:17" ht="84" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A16" s="95"/>
-      <c r="B16" s="142"/>
-      <c r="C16" s="65" t="s">
+      <c r="A16" s="91"/>
+      <c r="B16" s="145"/>
+      <c r="C16" s="64" t="s">
         <v>28</v>
       </c>
       <c r="D16" s="8" t="str">
@@ -2461,7 +2464,7 @@
 Team Analysis &amp; Design Model
 Team Git Set-Up</v>
       </c>
-      <c r="E16" s="51" t="s">
+      <c r="E16" s="50" t="s">
         <v>25</v>
       </c>
       <c r="F16" s="8" t="str">
@@ -2470,13 +2473,13 @@
 Team Analysis &amp; Design Model
 Team Git Set-Up</v>
       </c>
-      <c r="G16" s="133" t="s">
-        <v>43</v>
-      </c>
-      <c r="H16" s="51" t="s">
-        <v>47</v>
-      </c>
-      <c r="I16" s="139"/>
+      <c r="G16" s="128" t="s">
+        <v>42</v>
+      </c>
+      <c r="H16" s="50" t="s">
+        <v>46</v>
+      </c>
+      <c r="I16" s="134"/>
     </row>
     <row r="17" spans="1:17" ht="6.4" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B17" s="21"/>
@@ -2493,7 +2496,7 @@
       <c r="C18" s="30" t="s">
         <v>18</v>
       </c>
-      <c r="D18" s="57" t="s">
+      <c r="D18" s="56" t="s">
         <v>14</v>
       </c>
       <c r="E18" s="27" t="s">
@@ -2502,40 +2505,40 @@
       <c r="F18" s="28" t="s">
         <v>15</v>
       </c>
-      <c r="G18" s="82" t="s">
+      <c r="G18" s="80" t="s">
         <v>36</v>
       </c>
       <c r="H18" s="29" t="s">
         <v>16</v>
       </c>
-      <c r="I18" s="138" t="s">
-        <v>71</v>
+      <c r="I18" s="133" t="s">
+        <v>69</v>
       </c>
     </row>
     <row r="19" spans="1:17" ht="34.5" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B19" s="21"/>
       <c r="C19" s="30"/>
-      <c r="D19" s="79"/>
+      <c r="D19" s="77"/>
       <c r="E19" s="22"/>
-      <c r="F19" s="79"/>
+      <c r="F19" s="77"/>
       <c r="G19" s="22"/>
-      <c r="H19" s="79"/>
-      <c r="I19" s="79"/>
+      <c r="H19" s="77"/>
+      <c r="I19" s="77"/>
     </row>
     <row r="20" spans="1:17" ht="54" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A20" s="145" t="str">
+      <c r="A20" s="146" t="str">
         <f>A1</f>
         <v>CS320: SW Engineering - Spring 2025 Schedule
-(as of 1-6-2025, subject to change)</v>
-      </c>
-      <c r="B20" s="146"/>
-      <c r="C20" s="146"/>
-      <c r="D20" s="146"/>
-      <c r="E20" s="146"/>
-      <c r="F20" s="146"/>
-      <c r="G20" s="146"/>
-      <c r="H20" s="146"/>
-      <c r="I20" s="147"/>
+(as of 1-25-2025, subject to change)</v>
+      </c>
+      <c r="B20" s="147"/>
+      <c r="C20" s="147"/>
+      <c r="D20" s="147"/>
+      <c r="E20" s="147"/>
+      <c r="F20" s="147"/>
+      <c r="G20" s="147"/>
+      <c r="H20" s="147"/>
+      <c r="I20" s="148"/>
     </row>
     <row r="21" spans="1:17" s="2" customFormat="1" ht="17.25" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A21" s="1" t="str">
@@ -2544,43 +2547,43 @@
       </c>
       <c r="B21" s="1"/>
       <c r="C21" s="1" t="str">
-        <f>C2</f>
+        <f t="shared" ref="C21:I21" si="4">C2</f>
         <v>Sunday</v>
       </c>
       <c r="D21" s="1" t="str">
-        <f>D2</f>
+        <f t="shared" si="4"/>
         <v>Monday</v>
       </c>
       <c r="E21" s="1" t="str">
-        <f>E2</f>
+        <f t="shared" si="4"/>
         <v>Tuesday</v>
       </c>
       <c r="F21" s="1" t="str">
-        <f>F2</f>
+        <f t="shared" si="4"/>
         <v>Wednesday</v>
       </c>
       <c r="G21" s="1" t="str">
-        <f>G2</f>
+        <f t="shared" si="4"/>
         <v>Thursday</v>
       </c>
       <c r="H21" s="1" t="str">
-        <f>H2</f>
+        <f t="shared" si="4"/>
         <v>Friday</v>
       </c>
       <c r="I21" s="1" t="str">
-        <f>I2</f>
+        <f t="shared" si="4"/>
         <v>Saturday</v>
       </c>
     </row>
     <row r="22" spans="1:17" ht="15.75" customHeight="1" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="93">
+      <c r="A22" s="89">
         <f>A15-1</f>
         <v>8</v>
       </c>
-      <c r="B22" s="140" t="s">
+      <c r="B22" s="143" t="s">
         <v>11</v>
       </c>
-      <c r="C22" s="68">
+      <c r="C22" s="67">
         <f>I15 + 1</f>
         <v>16</v>
       </c>
@@ -2589,41 +2592,41 @@
         <v>17</v>
       </c>
       <c r="E22" s="16">
-        <f t="shared" ref="E22:I22" si="4">D22 + 1</f>
+        <f t="shared" ref="E22:I22" si="5">D22 + 1</f>
         <v>18</v>
       </c>
       <c r="F22" s="16">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>19</v>
       </c>
       <c r="G22" s="16">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>20</v>
       </c>
       <c r="H22" s="16">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>21</v>
       </c>
       <c r="I22" s="17">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>22</v>
       </c>
-      <c r="K22" s="79"/>
-      <c r="L22" s="77"/>
-      <c r="M22" s="77"/>
-      <c r="N22" s="77"/>
-      <c r="O22" s="77"/>
-      <c r="P22" s="77"/>
-      <c r="Q22" s="77"/>
+      <c r="K22" s="77"/>
+      <c r="L22" s="75"/>
+      <c r="M22" s="75"/>
+      <c r="N22" s="75"/>
+      <c r="O22" s="75"/>
+      <c r="P22" s="75"/>
+      <c r="Q22" s="75"/>
     </row>
     <row r="23" spans="1:17" ht="59.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="94"/>
-      <c r="B23" s="141"/>
-      <c r="C23" s="91"/>
+      <c r="A23" s="90"/>
+      <c r="B23" s="144"/>
+      <c r="C23" s="87"/>
       <c r="D23" s="6" t="s">
-        <v>46</v>
-      </c>
-      <c r="E23" s="44"/>
+        <v>45</v>
+      </c>
+      <c r="E23" s="43"/>
       <c r="F23" s="6" t="str">
         <f>D23</f>
         <v>Team Session: Final Preparation for Milestone 1
@@ -2634,20 +2637,20 @@
         <v>13</v>
       </c>
       <c r="I23" s="31"/>
-      <c r="K23" s="77"/>
-      <c r="L23" s="77"/>
-      <c r="M23" s="77"/>
-      <c r="N23" s="77"/>
-      <c r="O23" s="77"/>
-      <c r="P23" s="77"/>
+      <c r="K23" s="75"/>
+      <c r="L23" s="75"/>
+      <c r="M23" s="75"/>
+      <c r="N23" s="75"/>
+      <c r="O23" s="75"/>
+      <c r="P23" s="75"/>
       <c r="Q23" s="22"/>
     </row>
     <row r="24" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="94">
+      <c r="A24" s="90">
         <f>A22 - 1</f>
         <v>7</v>
       </c>
-      <c r="B24" s="141"/>
+      <c r="B24" s="144"/>
       <c r="C24" s="7">
         <f>I22 + 1</f>
         <v>23</v>
@@ -2657,72 +2660,72 @@
         <v>24</v>
       </c>
       <c r="E24" s="16">
-        <f t="shared" ref="E24:I24" si="5">D24 + 1</f>
+        <f t="shared" ref="E24:I24" si="6">D24 + 1</f>
         <v>25</v>
       </c>
       <c r="F24" s="16">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>26</v>
       </c>
       <c r="G24" s="16">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>27</v>
       </c>
       <c r="H24" s="16">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>28</v>
       </c>
       <c r="I24" s="17">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>29</v>
       </c>
-      <c r="K24" s="77"/>
-      <c r="L24" s="77"/>
-      <c r="M24" s="77"/>
-      <c r="N24" s="77"/>
-      <c r="O24" s="77"/>
-      <c r="P24" s="77"/>
-      <c r="Q24" s="77"/>
+      <c r="K24" s="75"/>
+      <c r="L24" s="75"/>
+      <c r="M24" s="75"/>
+      <c r="N24" s="75"/>
+      <c r="O24" s="75"/>
+      <c r="P24" s="75"/>
+      <c r="Q24" s="75"/>
     </row>
     <row r="25" spans="1:17" ht="129.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A25" s="94"/>
-      <c r="B25" s="141"/>
-      <c r="C25" s="76"/>
+      <c r="A25" s="90"/>
+      <c r="B25" s="144"/>
+      <c r="C25" s="74"/>
       <c r="D25" s="23" t="s">
         <v>22</v>
       </c>
-      <c r="E25" s="116"/>
-      <c r="F25" s="99" t="s">
+      <c r="E25" s="112"/>
+      <c r="F25" s="95" t="s">
         <v>32</v>
       </c>
-      <c r="G25" s="116"/>
-      <c r="H25" s="92" t="s">
-        <v>48</v>
-      </c>
-      <c r="I25" s="89"/>
+      <c r="G25" s="112"/>
+      <c r="H25" s="88" t="s">
+        <v>47</v>
+      </c>
+      <c r="I25" s="85"/>
       <c r="K25" s="22"/>
-      <c r="L25" s="77"/>
-      <c r="M25" s="79"/>
-      <c r="N25" s="77"/>
-      <c r="O25" s="79"/>
-      <c r="P25" s="77"/>
+      <c r="L25" s="75"/>
+      <c r="M25" s="77"/>
+      <c r="N25" s="75"/>
+      <c r="O25" s="77"/>
+      <c r="P25" s="75"/>
       <c r="Q25" s="22"/>
     </row>
     <row r="26" spans="1:17" ht="15" customHeight="1" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="154">
+      <c r="A26" s="151">
         <f>A24 - 1</f>
         <v>6</v>
       </c>
-      <c r="B26" s="97"/>
+      <c r="B26" s="93"/>
       <c r="C26" s="7">
         <f>I24 + 1</f>
         <v>30</v>
       </c>
-      <c r="D26" s="115">
+      <c r="D26" s="111">
         <f>C26 + 1</f>
         <v>31</v>
       </c>
-      <c r="E26" s="105">
+      <c r="E26" s="101">
         <f>IF(D26 = 31, 1, D36+1)</f>
         <v>1</v>
       </c>
@@ -2731,174 +2734,174 @@
         <v>2</v>
       </c>
       <c r="G26" s="33">
-        <f t="shared" ref="E26:G28" si="6">F26 + 1</f>
+        <f t="shared" ref="E26:G28" si="7">F26 + 1</f>
         <v>3</v>
       </c>
       <c r="H26" s="33">
-        <f t="shared" ref="H26" si="7">G26 + 1</f>
+        <f t="shared" ref="H26" si="8">G26 + 1</f>
         <v>4</v>
       </c>
-      <c r="I26" s="100">
-        <f t="shared" ref="I26" si="8">H26 + 1</f>
+      <c r="I26" s="96">
+        <f t="shared" ref="I26" si="9">H26 + 1</f>
         <v>5</v>
       </c>
-      <c r="K26" s="77"/>
-      <c r="L26" s="77"/>
-      <c r="M26" s="77"/>
-      <c r="N26" s="77"/>
-      <c r="O26" s="77"/>
-      <c r="P26" s="77"/>
-      <c r="Q26" s="77"/>
+      <c r="K26" s="75"/>
+      <c r="L26" s="75"/>
+      <c r="M26" s="75"/>
+      <c r="N26" s="75"/>
+      <c r="O26" s="75"/>
+      <c r="P26" s="75"/>
+      <c r="Q26" s="75"/>
     </row>
     <row r="27" spans="1:17" ht="68.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A27" s="150"/>
-      <c r="B27" s="98" t="s">
-        <v>59</v>
-      </c>
-      <c r="C27" s="49" t="s">
-        <v>78</v>
-      </c>
-      <c r="D27" s="81" t="s">
+      <c r="A27" s="138"/>
+      <c r="B27" s="94" t="s">
+        <v>57</v>
+      </c>
+      <c r="C27" s="48" t="s">
+        <v>74</v>
+      </c>
+      <c r="D27" s="79" t="s">
         <v>19</v>
       </c>
-      <c r="E27" s="118"/>
+      <c r="E27" s="114"/>
       <c r="F27" s="11" t="s">
-        <v>69</v>
-      </c>
-      <c r="G27" s="136"/>
-      <c r="H27" s="134" t="s">
-        <v>49</v>
-      </c>
-      <c r="I27" s="135" t="s">
+        <v>67</v>
+      </c>
+      <c r="G27" s="131"/>
+      <c r="H27" s="129" t="s">
+        <v>48</v>
+      </c>
+      <c r="I27" s="130" t="s">
         <v>34</v>
       </c>
-      <c r="K27" s="77"/>
-      <c r="L27" s="77"/>
+      <c r="K27" s="75"/>
+      <c r="L27" s="75"/>
       <c r="M27" s="22"/>
-      <c r="N27" s="77"/>
+      <c r="N27" s="75"/>
       <c r="O27" s="22"/>
-      <c r="P27" s="79"/>
+      <c r="P27" s="77"/>
       <c r="Q27" s="22"/>
     </row>
     <row r="28" spans="1:17" ht="15" customHeight="1" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="A28" s="155">
+      <c r="A28" s="152">
         <f>A26 -1</f>
         <v>5</v>
       </c>
-      <c r="B28" s="143" t="s">
+      <c r="B28" s="150" t="s">
         <v>12</v>
       </c>
       <c r="C28" s="12">
         <f>I26 + 1</f>
         <v>6</v>
       </c>
-      <c r="D28" s="42">
+      <c r="D28" s="41">
         <f>C28+1</f>
         <v>7</v>
       </c>
       <c r="E28" s="13">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>8</v>
       </c>
-      <c r="F28" s="42">
+      <c r="F28" s="41">
         <f>E28 + 1</f>
         <v>9</v>
       </c>
-      <c r="G28" s="38">
-        <f t="shared" si="6"/>
+      <c r="G28" s="37">
+        <f t="shared" si="7"/>
         <v>10</v>
       </c>
       <c r="H28" s="13">
         <f>G28 + 1</f>
         <v>11</v>
       </c>
-      <c r="I28" s="47">
+      <c r="I28" s="46">
         <f>H28 + 1</f>
         <v>12</v>
       </c>
     </row>
     <row r="29" spans="1:17" ht="55.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A29" s="156"/>
-      <c r="B29" s="144"/>
+      <c r="A29" s="153"/>
+      <c r="B29" s="141"/>
       <c r="C29" s="15"/>
       <c r="D29" s="9" t="s">
-        <v>79</v>
-      </c>
-      <c r="E29" s="40" t="s">
-        <v>70</v>
-      </c>
-      <c r="F29" s="39" t="s">
-        <v>52</v>
+        <v>75</v>
+      </c>
+      <c r="E29" s="39" t="s">
+        <v>68</v>
+      </c>
+      <c r="F29" s="38" t="s">
+        <v>51</v>
       </c>
       <c r="G29" s="24"/>
       <c r="H29" s="11" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="I29" s="25"/>
     </row>
     <row r="30" spans="1:17" ht="15.75" customHeight="1" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="A30" s="151">
+      <c r="A30" s="149">
         <f>A28 -1</f>
         <v>4</v>
       </c>
-      <c r="B30" s="144"/>
-      <c r="C30" s="48">
+      <c r="B30" s="141"/>
+      <c r="C30" s="47">
         <f>I28 + 1</f>
         <v>13</v>
       </c>
-      <c r="D30" s="38">
+      <c r="D30" s="37">
         <f>C30 + 1</f>
         <v>14</v>
       </c>
       <c r="E30" s="13">
-        <f t="shared" ref="E30:I30" si="9">D30 + 1</f>
+        <f t="shared" ref="E30:I30" si="10">D30 + 1</f>
         <v>15</v>
       </c>
       <c r="F30" s="13">
-        <f t="shared" si="9"/>
+        <f t="shared" si="10"/>
         <v>16</v>
       </c>
-      <c r="G30" s="38">
-        <f t="shared" si="9"/>
+      <c r="G30" s="37">
+        <f t="shared" si="10"/>
         <v>17</v>
       </c>
       <c r="H30" s="24">
-        <f t="shared" si="9"/>
+        <f t="shared" si="10"/>
         <v>18</v>
       </c>
       <c r="I30" s="25">
-        <f t="shared" si="9"/>
+        <f t="shared" si="10"/>
         <v>19</v>
       </c>
     </row>
     <row r="31" spans="1:17" ht="92.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A31" s="153"/>
-      <c r="B31" s="144"/>
+      <c r="A31" s="135"/>
+      <c r="B31" s="141"/>
       <c r="C31" s="26"/>
-      <c r="D31" s="74" t="s">
+      <c r="D31" s="73" t="s">
         <v>23</v>
       </c>
-      <c r="E31" s="75" t="s">
-        <v>77</v>
-      </c>
-      <c r="F31" s="39" t="s">
+      <c r="E31" s="159" t="s">
+        <v>80</v>
+      </c>
+      <c r="F31" s="23" t="s">
         <v>33</v>
       </c>
       <c r="G31" s="24"/>
-      <c r="H31" s="56" t="s">
+      <c r="H31" s="55" t="s">
         <v>30</v>
       </c>
-      <c r="I31" s="119" t="str">
+      <c r="I31" s="115" t="str">
         <f>H31</f>
         <v>Spring Break</v>
       </c>
     </row>
     <row r="32" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A32" s="153">
+      <c r="A32" s="135">
         <f>A30 -1</f>
         <v>3</v>
       </c>
-      <c r="B32" s="144"/>
+      <c r="B32" s="141"/>
       <c r="C32" s="24">
         <f>I30 + 1</f>
         <v>20</v>
@@ -2912,49 +2915,49 @@
         <v>22</v>
       </c>
       <c r="F32" s="13">
-        <f t="shared" ref="F32:I32" si="10">E32 + 1</f>
+        <f t="shared" ref="F32:I32" si="11">E32 + 1</f>
         <v>23</v>
       </c>
       <c r="G32" s="24">
-        <f t="shared" si="10"/>
+        <f t="shared" si="11"/>
         <v>24</v>
       </c>
       <c r="H32" s="24">
-        <f t="shared" si="10"/>
+        <f t="shared" si="11"/>
         <v>25</v>
       </c>
       <c r="I32" s="25">
-        <f t="shared" si="10"/>
+        <f t="shared" si="11"/>
         <v>26</v>
       </c>
     </row>
     <row r="33" spans="1:9" ht="52.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A33" s="153"/>
-      <c r="B33" s="144"/>
-      <c r="C33" s="55" t="str">
+      <c r="A33" s="135"/>
+      <c r="B33" s="141"/>
+      <c r="C33" s="54" t="str">
         <f>I31</f>
         <v>Spring Break</v>
       </c>
-      <c r="D33" s="126" t="str">
+      <c r="D33" s="122" t="str">
         <f>I31</f>
         <v>Spring Break</v>
       </c>
       <c r="E33" s="10"/>
-      <c r="F33" s="37" t="s">
-        <v>50</v>
-      </c>
-      <c r="G33" s="121"/>
-      <c r="H33" s="37" t="s">
-        <v>72</v>
-      </c>
-      <c r="I33" s="122"/>
+      <c r="F33" s="36" t="s">
+        <v>49</v>
+      </c>
+      <c r="G33" s="117"/>
+      <c r="H33" s="36" t="s">
+        <v>70</v>
+      </c>
+      <c r="I33" s="118"/>
     </row>
     <row r="34" spans="1:9" ht="15" customHeight="1" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="A34" s="153">
+      <c r="A34" s="135">
         <f>A32 -1</f>
         <v>2</v>
       </c>
-      <c r="B34" s="144" t="s">
+      <c r="B34" s="141" t="s">
         <v>29</v>
       </c>
       <c r="C34" s="26">
@@ -2966,52 +2969,52 @@
         <v>28</v>
       </c>
       <c r="E34" s="11">
-        <f t="shared" ref="E34:I36" si="11">D34 + 1</f>
+        <f t="shared" ref="E34:I36" si="12">D34 + 1</f>
         <v>29</v>
       </c>
-      <c r="F34" s="107">
-        <f t="shared" si="11"/>
+      <c r="F34" s="103">
+        <f t="shared" si="12"/>
         <v>30</v>
       </c>
-      <c r="G34" s="117">
+      <c r="G34" s="113">
         <f>IF(F34=30, 1, F34+1)</f>
         <v>1</v>
       </c>
       <c r="H34" s="4">
-        <f t="shared" si="11"/>
+        <f t="shared" si="12"/>
         <v>2</v>
       </c>
       <c r="I34" s="5">
-        <f t="shared" si="11"/>
+        <f t="shared" si="12"/>
         <v>3</v>
       </c>
     </row>
     <row r="35" spans="1:9" ht="58.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A35" s="152"/>
-      <c r="B35" s="148"/>
-      <c r="C35" s="46"/>
-      <c r="D35" s="36" t="s">
+      <c r="A35" s="136"/>
+      <c r="B35" s="142"/>
+      <c r="C35" s="45"/>
+      <c r="D35" s="35" t="s">
         <v>20</v>
       </c>
-      <c r="E35" s="35"/>
-      <c r="F35" s="120" t="s">
+      <c r="E35" s="34"/>
+      <c r="F35" s="116" t="s">
         <v>6</v>
       </c>
-      <c r="G35" s="123"/>
+      <c r="G35" s="119"/>
       <c r="H35" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="I35" s="125"/>
+      <c r="I35" s="121"/>
     </row>
     <row r="36" spans="1:9" ht="15" customHeight="1" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="A36" s="149">
+      <c r="A36" s="137">
         <f>A34 -1</f>
         <v>1</v>
       </c>
-      <c r="B36" s="140" t="s">
+      <c r="B36" s="143" t="s">
         <v>5</v>
       </c>
-      <c r="C36" s="117">
+      <c r="C36" s="113">
         <f>I34 + 1</f>
         <v>4</v>
       </c>
@@ -3020,11 +3023,11 @@
         <v>5</v>
       </c>
       <c r="E36" s="4">
-        <f t="shared" si="11"/>
+        <f t="shared" si="12"/>
         <v>6</v>
       </c>
-      <c r="F36" s="69">
-        <f t="shared" si="11"/>
+      <c r="F36" s="68">
+        <f t="shared" si="12"/>
         <v>7</v>
       </c>
       <c r="G36" s="16">
@@ -3036,94 +3039,83 @@
         <v>9</v>
       </c>
       <c r="I36" s="17">
-        <f t="shared" si="11"/>
+        <f t="shared" si="12"/>
         <v>10</v>
       </c>
     </row>
     <row r="37" spans="1:9" ht="90" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A37" s="150"/>
-      <c r="B37" s="141"/>
-      <c r="C37" s="76"/>
+      <c r="A37" s="138"/>
+      <c r="B37" s="144"/>
+      <c r="C37" s="74"/>
       <c r="D37" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="E37" s="124"/>
-      <c r="F37" s="70" t="s">
+      <c r="E37" s="120"/>
+      <c r="F37" s="69" t="s">
         <v>26</v>
       </c>
       <c r="G37" s="6"/>
       <c r="H37" s="6" t="s">
-        <v>56</v>
-      </c>
-      <c r="I37" s="135" t="s">
-        <v>53</v>
+        <v>54</v>
+      </c>
+      <c r="I37" s="130" t="s">
+        <v>52</v>
       </c>
     </row>
     <row r="38" spans="1:9" ht="15.75" customHeight="1" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="A38" s="157" t="s">
+      <c r="A38" s="139" t="s">
         <v>24</v>
       </c>
-      <c r="B38" s="141"/>
+      <c r="B38" s="144"/>
       <c r="C38" s="18">
         <f>I36 + 1</f>
         <v>11</v>
       </c>
       <c r="D38" s="16">
-        <f t="shared" ref="D38:I38" si="12">C38 + 1</f>
+        <f t="shared" ref="D38:I38" si="13">C38 + 1</f>
         <v>12</v>
       </c>
-      <c r="E38" s="45">
-        <f t="shared" si="12"/>
+      <c r="E38" s="44">
+        <f t="shared" si="13"/>
         <v>13</v>
       </c>
       <c r="F38" s="16">
-        <f t="shared" si="12"/>
+        <f t="shared" si="13"/>
         <v>14</v>
       </c>
       <c r="G38" s="16">
-        <f t="shared" si="12"/>
+        <f t="shared" si="13"/>
         <v>15</v>
       </c>
-      <c r="H38" s="58">
-        <f t="shared" si="12"/>
+      <c r="H38" s="57">
+        <f t="shared" si="13"/>
         <v>16</v>
       </c>
-      <c r="I38" s="59">
-        <f t="shared" si="12"/>
+      <c r="I38" s="58">
+        <f t="shared" si="13"/>
         <v>17</v>
       </c>
     </row>
     <row r="39" spans="1:9" ht="103.9" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A39" s="158"/>
-      <c r="B39" s="142"/>
-      <c r="C39" s="96"/>
+      <c r="A39" s="140"/>
+      <c r="B39" s="145"/>
+      <c r="C39" s="92"/>
       <c r="D39" s="20" t="s">
-        <v>57</v>
-      </c>
-      <c r="E39" s="50"/>
+        <v>55</v>
+      </c>
+      <c r="E39" s="49"/>
       <c r="F39" s="20" t="s">
-        <v>58</v>
-      </c>
-      <c r="G39" s="86" t="s">
-        <v>54</v>
-      </c>
-      <c r="H39" s="60"/>
-      <c r="I39" s="61"/>
+        <v>56</v>
+      </c>
+      <c r="G39" s="83" t="s">
+        <v>53</v>
+      </c>
+      <c r="H39" s="59"/>
+      <c r="I39" s="60"/>
     </row>
     <row r="40" spans="1:9" ht="15.75" thickTop="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <mergeCells count="22">
-    <mergeCell ref="A34:A35"/>
-    <mergeCell ref="A36:A37"/>
-    <mergeCell ref="A38:A39"/>
-    <mergeCell ref="B34:B35"/>
-    <mergeCell ref="B36:B39"/>
-    <mergeCell ref="A1:I1"/>
-    <mergeCell ref="A3:A4"/>
-    <mergeCell ref="A5:A6"/>
-    <mergeCell ref="A7:A8"/>
-    <mergeCell ref="A9:A10"/>
-    <mergeCell ref="B3:B4"/>
     <mergeCell ref="B13:B16"/>
     <mergeCell ref="B22:B25"/>
     <mergeCell ref="B28:B33"/>
@@ -3135,6 +3127,17 @@
     <mergeCell ref="A28:A29"/>
     <mergeCell ref="A30:A31"/>
     <mergeCell ref="A32:A33"/>
+    <mergeCell ref="A1:I1"/>
+    <mergeCell ref="A3:A4"/>
+    <mergeCell ref="A5:A6"/>
+    <mergeCell ref="A7:A8"/>
+    <mergeCell ref="A9:A10"/>
+    <mergeCell ref="B3:B4"/>
+    <mergeCell ref="A34:A35"/>
+    <mergeCell ref="A36:A37"/>
+    <mergeCell ref="A38:A39"/>
+    <mergeCell ref="B34:B35"/>
+    <mergeCell ref="B36:B39"/>
   </mergeCells>
   <printOptions horizontalCentered="1" verticalCentered="1"/>
   <pageMargins left="0.25" right="0.25" top="0.25" bottom="0.25" header="0" footer="0"/>

</xml_diff>

<commit_message>
updates to get things to match
</commit_message>
<xml_diff>
--- a/CS320-Spring2025Calendar.xlsx
+++ b/CS320-Spring2025Calendar.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\cygwin64\home\donha\cs320-spring2025\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{32F16F28-CA49-4963-AD2D-27275D190D10}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{18AABD3F-071A-45C0-9CEA-CF0EE58AA269}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="14940" yWindow="915" windowWidth="13665" windowHeight="14265" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -267,27 +267,6 @@
   </si>
   <si>
     <t>Assign06: Team Problem Domain Analysis Submission Review</t>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">Lecture  15: ORM, Designing a Persistence Layer
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="9"/>
-        <color rgb="FFFF0000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Lab 6: ORM
-(assigned)
-Lab 4: SQL
-due by 10:00a
-(Marmoset)</t>
-    </r>
   </si>
   <si>
     <t>A03: Team MS2
@@ -434,12 +413,6 @@
 (in-class)</t>
   </si>
   <si>
-    <t>Lab 6: ORM
-due  before class
---------&gt;&gt;&gt;
-(Marmoset)</t>
-  </si>
-  <si>
     <t>TBD (too be determined)</t>
   </si>
   <si>
@@ -448,41 +421,9 @@
 (in class)</t>
   </si>
   <si>
-    <r>
-      <t xml:space="preserve">Project Intros and Schedules
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="9"/>
-        <color rgb="FFFF0000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-Lab 0: ChatGPT
-due 7:00am
-(Marmoset)</t>
-    </r>
-  </si>
-  <si>
     <t>Prep Exam
 due Weds before class
 -------&gt;&gt;&gt;&gt;
-(Marmoset)</t>
-  </si>
-  <si>
-    <t>Lab 1: HTML &amp; CSS  Resume
-due Weds before class
---------&gt;&gt;&gt;&gt;
-(Marmoset)</t>
-  </si>
-  <si>
-    <t>Lab 5: JDBC
-due Mon before class
--------------&gt;&gt;&gt;&gt;
 (Marmoset)</t>
   </si>
   <si>
@@ -513,13 +454,6 @@
 (Marmoset)</t>
   </si>
   <si>
-    <t xml:space="preserve">Lab 2a: Web Apps Lab02a due
-Noon
-(after sign-off)
-(Marmoset)
-</t>
-  </si>
-  <si>
     <t>CS320: SW Engineering - Spring 2025 Schedule
 (as of 1-25-2025, subject to change)</t>
   </si>
@@ -529,6 +463,72 @@
 due Weds by Noon
 -----&gt;&gt;&gt;&gt;&gt;
 (Marmoset)</t>
+  </si>
+  <si>
+    <t>Lab 1: HTML &amp; CSS  Resume
+due Weds by Noon
+--------&gt;&gt;&gt;&gt;
+(Marmoset)</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Lecture  15: ORM, Designing a Persistence Layer
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="9"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Lab 6: ORM
+(assigned)
+Lab 4: SQL
+due by Noon
+(Marmoset)</t>
+    </r>
+  </si>
+  <si>
+    <t>Lab 5: JDBC
+due Mon by Noon
+-------------&gt;&gt;&gt;&gt;
+(Marmoset)</t>
+  </si>
+  <si>
+    <t>Lab 6: ORM
+due  by Noon
+--------&gt;&gt;&gt;
+(Marmoset)</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Project Intros and Schedules
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="9"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+Lab 0: ChatGPT
+due by Noon
+(Marmoset)</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">Lab 2a: Web Apps Lab02a due
+by Noon
+(after sign-off)
+(Marmoset)
+</t>
   </si>
 </sst>
 </file>
@@ -2001,7 +2001,7 @@
   <sheetData>
     <row r="1" spans="1:17" ht="53.1" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1" s="146" t="s">
-        <v>79</v>
+        <v>73</v>
       </c>
       <c r="B1" s="147"/>
       <c r="C1" s="147"/>
@@ -2044,7 +2044,7 @@
         <v>15</v>
       </c>
       <c r="B3" s="143" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="C3" s="52">
         <v>26</v>
@@ -2081,13 +2081,13 @@
         <v>7</v>
       </c>
       <c r="D4" s="95" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="E4" s="86" t="s">
-        <v>72</v>
+        <v>69</v>
       </c>
       <c r="F4" s="123" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="G4" s="32"/>
       <c r="H4" s="124" t="s">
@@ -2137,17 +2137,17 @@
       <c r="B6" s="141"/>
       <c r="C6" s="125"/>
       <c r="D6" s="38" t="s">
-        <v>71</v>
+        <v>79</v>
       </c>
       <c r="E6" s="39" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="F6" s="38" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="G6" s="61"/>
       <c r="H6" s="38" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="I6" s="71"/>
     </row>
@@ -2201,7 +2201,7 @@
       </c>
       <c r="G8" s="24"/>
       <c r="H8" s="132" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="I8" s="81"/>
     </row>
@@ -2251,21 +2251,21 @@
       <c r="A10" s="135"/>
       <c r="B10" s="141"/>
       <c r="C10" s="72" t="s">
-        <v>77</v>
+        <v>72</v>
       </c>
       <c r="D10" s="9" t="s">
         <v>39</v>
       </c>
       <c r="E10" s="61"/>
       <c r="F10" s="9" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="G10" s="10"/>
       <c r="H10" s="9" t="s">
         <v>27</v>
       </c>
       <c r="I10" s="157" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="K10" s="22"/>
       <c r="L10" s="75"/>
@@ -2281,7 +2281,7 @@
         <v>11</v>
       </c>
       <c r="B11" s="150" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="C11" s="15">
         <f>I9 + 1</f>
@@ -2394,11 +2394,11 @@
         <v>41</v>
       </c>
       <c r="D14" s="82" t="s">
-        <v>76</v>
+        <v>71</v>
       </c>
       <c r="E14" s="108"/>
       <c r="F14" s="6" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="G14" s="51" t="s">
         <v>28</v>
@@ -2512,7 +2512,7 @@
         <v>16</v>
       </c>
       <c r="I18" s="133" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
     </row>
     <row r="19" spans="1:17" ht="34.5" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -2700,7 +2700,7 @@
       </c>
       <c r="G25" s="112"/>
       <c r="H25" s="88" t="s">
-        <v>47</v>
+        <v>76</v>
       </c>
       <c r="I25" s="85"/>
       <c r="K25" s="22"/>
@@ -2756,21 +2756,21 @@
     <row r="27" spans="1:17" ht="68.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A27" s="138"/>
       <c r="B27" s="94" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="C27" s="48" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
       <c r="D27" s="79" t="s">
         <v>19</v>
       </c>
       <c r="E27" s="114"/>
       <c r="F27" s="11" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="G27" s="131"/>
       <c r="H27" s="129" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="I27" s="130" t="s">
         <v>34</v>
@@ -2825,17 +2825,17 @@
       <c r="B29" s="141"/>
       <c r="C29" s="15"/>
       <c r="D29" s="9" t="s">
-        <v>75</v>
+        <v>70</v>
       </c>
       <c r="E29" s="39" t="s">
-        <v>68</v>
+        <v>78</v>
       </c>
       <c r="F29" s="38" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="G29" s="24"/>
       <c r="H29" s="11" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="I29" s="25"/>
     </row>
@@ -2882,7 +2882,7 @@
         <v>23</v>
       </c>
       <c r="E31" s="159" t="s">
-        <v>80</v>
+        <v>74</v>
       </c>
       <c r="F31" s="23" t="s">
         <v>33</v>
@@ -2944,11 +2944,11 @@
       </c>
       <c r="E33" s="10"/>
       <c r="F33" s="36" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="G33" s="117"/>
       <c r="H33" s="36" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="I33" s="118"/>
     </row>
@@ -3056,10 +3056,10 @@
       </c>
       <c r="G37" s="6"/>
       <c r="H37" s="6" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="I37" s="130" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
     </row>
     <row r="38" spans="1:9" ht="15.75" customHeight="1" thickTop="1" x14ac:dyDescent="0.25">
@@ -3101,14 +3101,14 @@
       <c r="B39" s="145"/>
       <c r="C39" s="92"/>
       <c r="D39" s="20" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="E39" s="49"/>
       <c r="F39" s="20" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="G39" s="83" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="H39" s="59"/>
       <c r="I39" s="60"/>

</xml_diff>

<commit_message>
updated news and schedule
</commit_message>
<xml_diff>
--- a/CS320-Spring2025Calendar.xlsx
+++ b/CS320-Spring2025Calendar.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\cygwin64\home\donha\cs320-spring2025\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C64E44DB-A5C8-417C-AD47-EAFB2BB82560}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1F25D98C-6C5D-4CA2-9B6D-70FB39CEC632}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3420" yWindow="0" windowWidth="20790" windowHeight="14865" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="345" yWindow="570" windowWidth="24345" windowHeight="14730" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Calendar-Sp24" sheetId="1" r:id="rId1"/>
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="88" uniqueCount="82">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="88" uniqueCount="83">
   <si>
     <t>Monday</t>
   </si>
@@ -509,10 +509,6 @@
     <t>Team Project Introduction and  Schedule</t>
   </si>
   <si>
-    <t>CS320: SW Engineering - Spring 2025 Schedule
-(as of 2-11-2025, subject to change)</t>
-  </si>
-  <si>
     <r>
       <t xml:space="preserve">Lecture 4: Web Applications
 </t>
@@ -549,6 +545,31 @@
       <t>Lab02: Web App Introduction due
 (in class)</t>
     </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Winter
+Break
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="9"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Lab 2a: Web Apps Lab02a resubmissions due
+by Noon
+(after sign-off)
+(Marmoset)</t>
+    </r>
+  </si>
+  <si>
+    <t>CS320: SW Engineering - Spring 2025 Schedule
+(as of 2-26-2025, subject to change)</t>
   </si>
 </sst>
 </file>
@@ -1211,7 +1232,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="158">
+  <cellXfs count="157">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -1420,9 +1441,6 @@
     <xf numFmtId="0" fontId="3" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="7" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1624,16 +1642,58 @@
     <xf numFmtId="0" fontId="7" fillId="4" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1641,48 +1701,6 @@
     </xf>
     <xf numFmtId="0" fontId="9" fillId="2" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -2011,17 +2029,17 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:17" ht="53.1" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="149" t="s">
-        <v>79</v>
-      </c>
-      <c r="B1" s="150"/>
-      <c r="C1" s="150"/>
-      <c r="D1" s="150"/>
-      <c r="E1" s="150"/>
-      <c r="F1" s="150"/>
-      <c r="G1" s="150"/>
-      <c r="H1" s="150"/>
-      <c r="I1" s="151"/>
+      <c r="A1" s="143" t="s">
+        <v>82</v>
+      </c>
+      <c r="B1" s="144"/>
+      <c r="C1" s="144"/>
+      <c r="D1" s="144"/>
+      <c r="E1" s="144"/>
+      <c r="F1" s="144"/>
+      <c r="G1" s="144"/>
+      <c r="H1" s="144"/>
+      <c r="I1" s="145"/>
     </row>
     <row r="2" spans="1:17" s="2" customFormat="1" ht="21" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
@@ -2043,7 +2061,7 @@
       <c r="G2" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="H2" s="97" t="s">
+      <c r="H2" s="96" t="s">
         <v>4</v>
       </c>
       <c r="I2" s="1" t="s">
@@ -2051,10 +2069,10 @@
       </c>
     </row>
     <row r="3" spans="1:17" ht="15.75" customHeight="1" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="140">
+      <c r="A3" s="154">
         <v>15</v>
       </c>
-      <c r="B3" s="146" t="s">
+      <c r="B3" s="138" t="s">
         <v>54</v>
       </c>
       <c r="C3" s="52">
@@ -2076,45 +2094,45 @@
         <f t="shared" si="0"/>
         <v>30</v>
       </c>
-      <c r="H3" s="98">
+      <c r="H3" s="97">
         <f t="shared" si="0"/>
         <v>31</v>
       </c>
-      <c r="I3" s="99">
+      <c r="I3" s="98">
         <f>IF(H3 = 31, 1, H3+1)</f>
         <v>1</v>
       </c>
     </row>
     <row r="4" spans="1:17" ht="101.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="141"/>
-      <c r="B4" s="148"/>
-      <c r="C4" s="100" t="s">
+      <c r="A4" s="150"/>
+      <c r="B4" s="140"/>
+      <c r="C4" s="99" t="s">
         <v>7</v>
       </c>
-      <c r="D4" s="95" t="s">
+      <c r="D4" s="94" t="s">
         <v>55</v>
       </c>
-      <c r="E4" s="86" t="s">
+      <c r="E4" s="85" t="s">
         <v>65</v>
       </c>
-      <c r="F4" s="123" t="s">
+      <c r="F4" s="122" t="s">
         <v>57</v>
       </c>
       <c r="G4" s="32"/>
-      <c r="H4" s="116" t="s">
+      <c r="H4" s="115" t="s">
         <v>74</v>
       </c>
-      <c r="I4" s="102"/>
+      <c r="I4" s="101"/>
     </row>
     <row r="5" spans="1:17" ht="15" customHeight="1" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="152">
+      <c r="A5" s="153">
         <f>A3 - 1</f>
         <v>14</v>
       </c>
-      <c r="B5" s="153" t="s">
+      <c r="B5" s="141" t="s">
         <v>10</v>
       </c>
-      <c r="C5" s="101">
+      <c r="C5" s="100">
         <f>I3 + 1</f>
         <v>2</v>
       </c>
@@ -2144,9 +2162,9 @@
       </c>
     </row>
     <row r="6" spans="1:17" ht="122.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="139"/>
-      <c r="B6" s="144"/>
-      <c r="C6" s="124"/>
+      <c r="A6" s="148"/>
+      <c r="B6" s="142"/>
+      <c r="C6" s="123"/>
       <c r="D6" s="38" t="s">
         <v>77</v>
       </c>
@@ -2162,14 +2180,14 @@
       <c r="H6" s="38" t="s">
         <v>58</v>
       </c>
-      <c r="I6" s="71"/>
+      <c r="I6" s="70"/>
     </row>
     <row r="7" spans="1:17" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="138">
+      <c r="A7" s="147">
         <f>A5 - 1</f>
         <v>13</v>
       </c>
-      <c r="B7" s="144"/>
+      <c r="B7" s="142"/>
       <c r="C7" s="15">
         <f>I5 + 1</f>
         <v>9</v>
@@ -2200,9 +2218,9 @@
       </c>
     </row>
     <row r="8" spans="1:17" ht="123.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="138"/>
-      <c r="B8" s="144"/>
-      <c r="C8" s="133" t="s">
+      <c r="A8" s="147"/>
+      <c r="B8" s="142"/>
+      <c r="C8" s="132" t="s">
         <v>31</v>
       </c>
       <c r="D8" s="38" t="s">
@@ -2210,20 +2228,20 @@
       </c>
       <c r="E8" s="61"/>
       <c r="F8" s="11" t="s">
+        <v>79</v>
+      </c>
+      <c r="G8" s="24"/>
+      <c r="H8" s="137" t="s">
         <v>80</v>
       </c>
-      <c r="G8" s="24"/>
-      <c r="H8" s="157" t="s">
-        <v>81</v>
-      </c>
-      <c r="I8" s="81"/>
+      <c r="I8" s="80"/>
     </row>
     <row r="9" spans="1:17" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="138">
+      <c r="A9" s="147">
         <f>A7 - 1</f>
         <v>12</v>
       </c>
-      <c r="B9" s="144"/>
+      <c r="B9" s="142"/>
       <c r="C9" s="12">
         <f>I7 + 1</f>
         <v>16</v>
@@ -2252,18 +2270,18 @@
         <f t="shared" si="1"/>
         <v>22</v>
       </c>
-      <c r="K9" s="75"/>
-      <c r="L9" s="75"/>
-      <c r="M9" s="75"/>
-      <c r="N9" s="75"/>
-      <c r="O9" s="75"/>
-      <c r="P9" s="75"/>
-      <c r="Q9" s="75"/>
+      <c r="K9" s="74"/>
+      <c r="L9" s="74"/>
+      <c r="M9" s="74"/>
+      <c r="N9" s="74"/>
+      <c r="O9" s="74"/>
+      <c r="P9" s="74"/>
+      <c r="Q9" s="74"/>
     </row>
     <row r="10" spans="1:17" ht="102.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="138"/>
-      <c r="B10" s="144"/>
-      <c r="C10" s="72" t="s">
+      <c r="A10" s="147"/>
+      <c r="B10" s="142"/>
+      <c r="C10" s="71" t="s">
         <v>68</v>
       </c>
       <c r="D10" s="9" t="s">
@@ -2277,23 +2295,23 @@
       <c r="H10" s="9" t="s">
         <v>27</v>
       </c>
-      <c r="I10" s="135" t="s">
+      <c r="I10" s="134" t="s">
         <v>73</v>
       </c>
       <c r="K10" s="22"/>
-      <c r="L10" s="75"/>
-      <c r="M10" s="76"/>
-      <c r="N10" s="75"/>
-      <c r="O10" s="76"/>
-      <c r="P10" s="75"/>
-      <c r="Q10" s="76"/>
+      <c r="L10" s="74"/>
+      <c r="M10" s="75"/>
+      <c r="N10" s="74"/>
+      <c r="O10" s="75"/>
+      <c r="P10" s="74"/>
+      <c r="Q10" s="75"/>
     </row>
     <row r="11" spans="1:17" ht="15" customHeight="1" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="138">
+      <c r="A11" s="147">
         <f>A9 -1</f>
         <v>11</v>
       </c>
-      <c r="B11" s="153" t="s">
+      <c r="B11" s="141" t="s">
         <v>56</v>
       </c>
       <c r="C11" s="15">
@@ -2316,55 +2334,55 @@
         <f t="shared" si="1"/>
         <v>27</v>
       </c>
-      <c r="H11" s="103">
+      <c r="H11" s="102">
         <f t="shared" si="1"/>
         <v>28</v>
       </c>
-      <c r="I11" s="109">
+      <c r="I11" s="108">
         <f>IF(H11 = 28,1,H11+1)</f>
         <v>1</v>
       </c>
-      <c r="K11" s="75"/>
-      <c r="L11" s="75"/>
-      <c r="M11" s="75"/>
-      <c r="N11" s="75"/>
-      <c r="O11" s="75"/>
-      <c r="P11" s="75"/>
-      <c r="Q11" s="75"/>
+      <c r="K11" s="74"/>
+      <c r="L11" s="74"/>
+      <c r="M11" s="74"/>
+      <c r="N11" s="74"/>
+      <c r="O11" s="74"/>
+      <c r="P11" s="74"/>
+      <c r="Q11" s="74"/>
     </row>
     <row r="12" spans="1:17" ht="120" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="139"/>
-      <c r="B12" s="145"/>
-      <c r="C12" s="134"/>
+      <c r="A12" s="148"/>
+      <c r="B12" s="146"/>
+      <c r="C12" s="133"/>
       <c r="D12" s="36" t="s">
         <v>41</v>
       </c>
-      <c r="E12" s="125"/>
-      <c r="F12" s="126" t="s">
+      <c r="E12" s="124"/>
+      <c r="F12" s="125" t="s">
         <v>40</v>
       </c>
       <c r="G12" s="34"/>
-      <c r="H12" s="137" t="s">
+      <c r="H12" s="136" t="s">
         <v>21</v>
       </c>
-      <c r="I12" s="110"/>
+      <c r="I12" s="109"/>
       <c r="K12" s="22"/>
-      <c r="L12" s="75"/>
-      <c r="M12" s="75"/>
-      <c r="N12" s="75"/>
-      <c r="O12" s="76"/>
-      <c r="P12" s="75"/>
-      <c r="Q12" s="76"/>
+      <c r="L12" s="74"/>
+      <c r="M12" s="74"/>
+      <c r="N12" s="74"/>
+      <c r="O12" s="75"/>
+      <c r="P12" s="74"/>
+      <c r="Q12" s="75"/>
     </row>
     <row r="13" spans="1:17" ht="15" customHeight="1" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="106">
+      <c r="A13" s="105">
         <f xml:space="preserve"> A11 - 1</f>
         <v>10</v>
       </c>
-      <c r="B13" s="146" t="s">
+      <c r="B13" s="138" t="s">
         <v>11</v>
       </c>
-      <c r="C13" s="107">
+      <c r="C13" s="106">
         <f>IF(I11=28, 1, I11+1)</f>
         <v>2</v>
       </c>
@@ -2392,50 +2410,50 @@
         <f t="shared" si="1"/>
         <v>8</v>
       </c>
-      <c r="K13" s="75"/>
-      <c r="L13" s="75"/>
-      <c r="M13" s="75"/>
-      <c r="N13" s="75"/>
-      <c r="O13" s="75"/>
-      <c r="P13" s="75"/>
-      <c r="Q13" s="77"/>
+      <c r="K13" s="74"/>
+      <c r="L13" s="74"/>
+      <c r="M13" s="74"/>
+      <c r="N13" s="74"/>
+      <c r="O13" s="74"/>
+      <c r="P13" s="74"/>
+      <c r="Q13" s="76"/>
     </row>
     <row r="14" spans="1:17" ht="144.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="105"/>
-      <c r="B14" s="147"/>
-      <c r="C14" s="84" t="s">
+      <c r="A14" s="104"/>
+      <c r="B14" s="139"/>
+      <c r="C14" s="83" t="s">
         <v>38</v>
       </c>
-      <c r="D14" s="82" t="s">
+      <c r="D14" s="81" t="s">
         <v>67</v>
       </c>
-      <c r="E14" s="108"/>
+      <c r="E14" s="107"/>
       <c r="F14" s="6" t="s">
         <v>61</v>
       </c>
       <c r="G14" s="51" t="s">
         <v>28</v>
       </c>
-      <c r="H14" s="70" t="s">
-        <v>28</v>
+      <c r="H14" s="38" t="s">
+        <v>81</v>
       </c>
       <c r="I14" s="63" t="s">
         <v>28</v>
       </c>
-      <c r="K14" s="77"/>
+      <c r="K14" s="76"/>
       <c r="L14" s="22"/>
-      <c r="M14" s="78"/>
-      <c r="N14" s="75"/>
-      <c r="O14" s="77"/>
-      <c r="P14" s="75"/>
-      <c r="Q14" s="77"/>
+      <c r="M14" s="77"/>
+      <c r="N14" s="74"/>
+      <c r="O14" s="76"/>
+      <c r="P14" s="74"/>
+      <c r="Q14" s="76"/>
     </row>
     <row r="15" spans="1:17" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="90">
+      <c r="A15" s="89">
         <f>A13 - 1</f>
         <v>9</v>
       </c>
-      <c r="B15" s="147"/>
+      <c r="B15" s="139"/>
       <c r="C15" s="54">
         <f>I13 + 1</f>
         <v>9</v>
@@ -2444,7 +2462,7 @@
         <f t="shared" ref="D15:I15" si="3">C15 + 1</f>
         <v>10</v>
       </c>
-      <c r="E15" s="82">
+      <c r="E15" s="81">
         <f t="shared" si="3"/>
         <v>11</v>
       </c>
@@ -2452,7 +2470,7 @@
         <f t="shared" si="3"/>
         <v>12</v>
       </c>
-      <c r="G15" s="104">
+      <c r="G15" s="103">
         <f t="shared" si="3"/>
         <v>13</v>
       </c>
@@ -2466,8 +2484,8 @@
       </c>
     </row>
     <row r="16" spans="1:17" ht="84" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A16" s="91"/>
-      <c r="B16" s="148"/>
+      <c r="A16" s="90"/>
+      <c r="B16" s="140"/>
       <c r="C16" s="64" t="s">
         <v>28</v>
       </c>
@@ -2486,13 +2504,13 @@
 Team Analysis &amp; Design Model
 Team Git Set-Up</v>
       </c>
-      <c r="G16" s="127" t="s">
+      <c r="G16" s="126" t="s">
         <v>39</v>
       </c>
       <c r="H16" s="50" t="s">
         <v>43</v>
       </c>
-      <c r="I16" s="132"/>
+      <c r="I16" s="131"/>
     </row>
     <row r="17" spans="1:17" ht="6.4" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B17" s="21"/>
@@ -2518,40 +2536,40 @@
       <c r="F18" s="28" t="s">
         <v>15</v>
       </c>
-      <c r="G18" s="80" t="s">
+      <c r="G18" s="79" t="s">
         <v>36</v>
       </c>
       <c r="H18" s="29" t="s">
         <v>16</v>
       </c>
-      <c r="I18" s="131" t="s">
+      <c r="I18" s="130" t="s">
         <v>63</v>
       </c>
     </row>
     <row r="19" spans="1:17" ht="34.5" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B19" s="21"/>
       <c r="C19" s="30"/>
-      <c r="D19" s="77"/>
+      <c r="D19" s="76"/>
       <c r="E19" s="22"/>
-      <c r="F19" s="77"/>
+      <c r="F19" s="76"/>
       <c r="G19" s="22"/>
-      <c r="H19" s="77"/>
-      <c r="I19" s="77"/>
+      <c r="H19" s="76"/>
+      <c r="I19" s="76"/>
     </row>
     <row r="20" spans="1:17" ht="54" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A20" s="149" t="str">
+      <c r="A20" s="143" t="str">
         <f>A1</f>
         <v>CS320: SW Engineering - Spring 2025 Schedule
-(as of 2-11-2025, subject to change)</v>
-      </c>
-      <c r="B20" s="150"/>
-      <c r="C20" s="150"/>
-      <c r="D20" s="150"/>
-      <c r="E20" s="150"/>
-      <c r="F20" s="150"/>
-      <c r="G20" s="150"/>
-      <c r="H20" s="150"/>
-      <c r="I20" s="151"/>
+(as of 2-26-2025, subject to change)</v>
+      </c>
+      <c r="B20" s="144"/>
+      <c r="C20" s="144"/>
+      <c r="D20" s="144"/>
+      <c r="E20" s="144"/>
+      <c r="F20" s="144"/>
+      <c r="G20" s="144"/>
+      <c r="H20" s="144"/>
+      <c r="I20" s="145"/>
     </row>
     <row r="21" spans="1:17" s="2" customFormat="1" ht="17.25" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A21" s="1" t="str">
@@ -2589,11 +2607,11 @@
       </c>
     </row>
     <row r="22" spans="1:17" ht="15.75" customHeight="1" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="89">
+      <c r="A22" s="88">
         <f>A15-1</f>
         <v>8</v>
       </c>
-      <c r="B22" s="146" t="s">
+      <c r="B22" s="138" t="s">
         <v>11</v>
       </c>
       <c r="C22" s="67">
@@ -2624,18 +2642,18 @@
         <f t="shared" si="5"/>
         <v>22</v>
       </c>
-      <c r="K22" s="77"/>
-      <c r="L22" s="75"/>
-      <c r="M22" s="75"/>
-      <c r="N22" s="75"/>
-      <c r="O22" s="75"/>
-      <c r="P22" s="75"/>
-      <c r="Q22" s="75"/>
+      <c r="K22" s="76"/>
+      <c r="L22" s="74"/>
+      <c r="M22" s="74"/>
+      <c r="N22" s="74"/>
+      <c r="O22" s="74"/>
+      <c r="P22" s="74"/>
+      <c r="Q22" s="74"/>
     </row>
     <row r="23" spans="1:17" ht="59.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="90"/>
-      <c r="B23" s="147"/>
-      <c r="C23" s="87"/>
+      <c r="A23" s="89"/>
+      <c r="B23" s="139"/>
+      <c r="C23" s="86"/>
       <c r="D23" s="6" t="s">
         <v>42</v>
       </c>
@@ -2650,20 +2668,20 @@
         <v>13</v>
       </c>
       <c r="I23" s="31"/>
-      <c r="K23" s="75"/>
-      <c r="L23" s="75"/>
-      <c r="M23" s="75"/>
-      <c r="N23" s="75"/>
-      <c r="O23" s="75"/>
-      <c r="P23" s="75"/>
+      <c r="K23" s="74"/>
+      <c r="L23" s="74"/>
+      <c r="M23" s="74"/>
+      <c r="N23" s="74"/>
+      <c r="O23" s="74"/>
+      <c r="P23" s="74"/>
       <c r="Q23" s="22"/>
     </row>
     <row r="24" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="90">
+      <c r="A24" s="89">
         <f>A22 - 1</f>
         <v>7</v>
       </c>
-      <c r="B24" s="147"/>
+      <c r="B24" s="139"/>
       <c r="C24" s="7">
         <f>I22 + 1</f>
         <v>23</v>
@@ -2692,53 +2710,53 @@
         <f t="shared" si="6"/>
         <v>29</v>
       </c>
-      <c r="K24" s="75"/>
-      <c r="L24" s="75"/>
-      <c r="M24" s="75"/>
-      <c r="N24" s="75"/>
-      <c r="O24" s="75"/>
-      <c r="P24" s="75"/>
-      <c r="Q24" s="75"/>
+      <c r="K24" s="74"/>
+      <c r="L24" s="74"/>
+      <c r="M24" s="74"/>
+      <c r="N24" s="74"/>
+      <c r="O24" s="74"/>
+      <c r="P24" s="74"/>
+      <c r="Q24" s="74"/>
     </row>
     <row r="25" spans="1:17" ht="129.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A25" s="90"/>
-      <c r="B25" s="147"/>
-      <c r="C25" s="74"/>
+      <c r="A25" s="89"/>
+      <c r="B25" s="139"/>
+      <c r="C25" s="73"/>
       <c r="D25" s="23" t="s">
         <v>22</v>
       </c>
-      <c r="E25" s="112"/>
-      <c r="F25" s="95" t="s">
+      <c r="E25" s="111"/>
+      <c r="F25" s="94" t="s">
         <v>32</v>
       </c>
-      <c r="G25" s="112"/>
-      <c r="H25" s="88" t="s">
+      <c r="G25" s="111"/>
+      <c r="H25" s="87" t="s">
         <v>70</v>
       </c>
-      <c r="I25" s="85"/>
+      <c r="I25" s="84"/>
       <c r="K25" s="22"/>
-      <c r="L25" s="75"/>
-      <c r="M25" s="77"/>
-      <c r="N25" s="75"/>
-      <c r="O25" s="77"/>
-      <c r="P25" s="75"/>
+      <c r="L25" s="74"/>
+      <c r="M25" s="76"/>
+      <c r="N25" s="74"/>
+      <c r="O25" s="76"/>
+      <c r="P25" s="74"/>
       <c r="Q25" s="22"/>
     </row>
     <row r="26" spans="1:17" ht="15" customHeight="1" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="154">
+      <c r="A26" s="149">
         <f>A24 - 1</f>
         <v>6</v>
       </c>
-      <c r="B26" s="93"/>
+      <c r="B26" s="92"/>
       <c r="C26" s="7">
         <f>I24 + 1</f>
         <v>30</v>
       </c>
-      <c r="D26" s="111">
+      <c r="D26" s="110">
         <f>C26 + 1</f>
         <v>31</v>
       </c>
-      <c r="E26" s="101">
+      <c r="E26" s="100">
         <f>IF(D26 = 31, 1, D36+1)</f>
         <v>1</v>
       </c>
@@ -2754,54 +2772,54 @@
         <f t="shared" ref="H26" si="8">G26 + 1</f>
         <v>4</v>
       </c>
-      <c r="I26" s="96">
+      <c r="I26" s="95">
         <f t="shared" ref="I26" si="9">H26 + 1</f>
         <v>5</v>
       </c>
-      <c r="K26" s="75"/>
-      <c r="L26" s="75"/>
-      <c r="M26" s="75"/>
-      <c r="N26" s="75"/>
-      <c r="O26" s="75"/>
-      <c r="P26" s="75"/>
-      <c r="Q26" s="75"/>
+      <c r="K26" s="74"/>
+      <c r="L26" s="74"/>
+      <c r="M26" s="74"/>
+      <c r="N26" s="74"/>
+      <c r="O26" s="74"/>
+      <c r="P26" s="74"/>
+      <c r="Q26" s="74"/>
     </row>
     <row r="27" spans="1:17" ht="68.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A27" s="141"/>
-      <c r="B27" s="94" t="s">
+      <c r="A27" s="150"/>
+      <c r="B27" s="93" t="s">
         <v>53</v>
       </c>
       <c r="C27" s="48" t="s">
         <v>71</v>
       </c>
-      <c r="D27" s="79" t="s">
+      <c r="D27" s="78" t="s">
         <v>19</v>
       </c>
-      <c r="E27" s="114"/>
+      <c r="E27" s="113"/>
       <c r="F27" s="11" t="s">
         <v>62</v>
       </c>
-      <c r="G27" s="130"/>
-      <c r="H27" s="128" t="s">
+      <c r="G27" s="129"/>
+      <c r="H27" s="127" t="s">
         <v>44</v>
       </c>
-      <c r="I27" s="129" t="s">
+      <c r="I27" s="128" t="s">
         <v>34</v>
       </c>
-      <c r="K27" s="75"/>
-      <c r="L27" s="75"/>
+      <c r="K27" s="74"/>
+      <c r="L27" s="74"/>
       <c r="M27" s="22"/>
-      <c r="N27" s="75"/>
+      <c r="N27" s="74"/>
       <c r="O27" s="22"/>
-      <c r="P27" s="77"/>
+      <c r="P27" s="76"/>
       <c r="Q27" s="22"/>
     </row>
     <row r="28" spans="1:17" ht="15" customHeight="1" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="A28" s="155">
+      <c r="A28" s="151">
         <f>A26 -1</f>
         <v>5</v>
       </c>
-      <c r="B28" s="153" t="s">
+      <c r="B28" s="141" t="s">
         <v>12</v>
       </c>
       <c r="C28" s="12">
@@ -2834,8 +2852,8 @@
       </c>
     </row>
     <row r="29" spans="1:17" ht="55.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A29" s="156"/>
-      <c r="B29" s="144"/>
+      <c r="A29" s="152"/>
+      <c r="B29" s="142"/>
       <c r="C29" s="15"/>
       <c r="D29" s="9" t="s">
         <v>66</v>
@@ -2853,11 +2871,11 @@
       <c r="I29" s="25"/>
     </row>
     <row r="30" spans="1:17" ht="15.75" customHeight="1" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="A30" s="152">
+      <c r="A30" s="153">
         <f>A28 -1</f>
         <v>4</v>
       </c>
-      <c r="B30" s="144"/>
+      <c r="B30" s="142"/>
       <c r="C30" s="47">
         <f>I28 + 1</f>
         <v>13</v>
@@ -2888,13 +2906,13 @@
       </c>
     </row>
     <row r="31" spans="1:17" ht="92.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A31" s="138"/>
-      <c r="B31" s="144"/>
+      <c r="A31" s="147"/>
+      <c r="B31" s="142"/>
       <c r="C31" s="26"/>
-      <c r="D31" s="73" t="s">
+      <c r="D31" s="72" t="s">
         <v>23</v>
       </c>
-      <c r="E31" s="136" t="s">
+      <c r="E31" s="135" t="s">
         <v>69</v>
       </c>
       <c r="F31" s="23" t="s">
@@ -2904,17 +2922,17 @@
       <c r="H31" s="55" t="s">
         <v>30</v>
       </c>
-      <c r="I31" s="115" t="str">
+      <c r="I31" s="114" t="str">
         <f>H31</f>
         <v>Spring Break</v>
       </c>
     </row>
     <row r="32" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A32" s="138">
+      <c r="A32" s="147">
         <f>A30 -1</f>
         <v>3</v>
       </c>
-      <c r="B32" s="144"/>
+      <c r="B32" s="142"/>
       <c r="C32" s="24">
         <f>I30 + 1</f>
         <v>20</v>
@@ -2945,13 +2963,13 @@
       </c>
     </row>
     <row r="33" spans="1:9" ht="52.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A33" s="138"/>
-      <c r="B33" s="144"/>
+      <c r="A33" s="147"/>
+      <c r="B33" s="142"/>
       <c r="C33" s="54" t="str">
         <f>I31</f>
         <v>Spring Break</v>
       </c>
-      <c r="D33" s="122" t="str">
+      <c r="D33" s="121" t="str">
         <f>I31</f>
         <v>Spring Break</v>
       </c>
@@ -2959,18 +2977,18 @@
       <c r="F33" s="36" t="s">
         <v>45</v>
       </c>
-      <c r="G33" s="117"/>
+      <c r="G33" s="116"/>
       <c r="H33" s="36" t="s">
         <v>64</v>
       </c>
-      <c r="I33" s="118"/>
+      <c r="I33" s="117"/>
     </row>
     <row r="34" spans="1:9" ht="15" customHeight="1" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="A34" s="138">
+      <c r="A34" s="147">
         <f>A32 -1</f>
         <v>2</v>
       </c>
-      <c r="B34" s="144" t="s">
+      <c r="B34" s="142" t="s">
         <v>29</v>
       </c>
       <c r="C34" s="26">
@@ -2985,11 +3003,11 @@
         <f t="shared" ref="E34:I36" si="12">D34 + 1</f>
         <v>29</v>
       </c>
-      <c r="F34" s="103">
+      <c r="F34" s="102">
         <f t="shared" si="12"/>
         <v>30</v>
       </c>
-      <c r="G34" s="113">
+      <c r="G34" s="112">
         <f>IF(F34=30, 1, F34+1)</f>
         <v>1</v>
       </c>
@@ -3003,31 +3021,31 @@
       </c>
     </row>
     <row r="35" spans="1:9" ht="58.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A35" s="139"/>
-      <c r="B35" s="145"/>
+      <c r="A35" s="148"/>
+      <c r="B35" s="146"/>
       <c r="C35" s="45"/>
       <c r="D35" s="35" t="s">
         <v>20</v>
       </c>
       <c r="E35" s="34"/>
-      <c r="F35" s="116" t="s">
+      <c r="F35" s="115" t="s">
         <v>6</v>
       </c>
-      <c r="G35" s="119"/>
+      <c r="G35" s="118"/>
       <c r="H35" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="I35" s="121"/>
+      <c r="I35" s="120"/>
     </row>
     <row r="36" spans="1:9" ht="15" customHeight="1" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="A36" s="140">
+      <c r="A36" s="154">
         <f>A34 -1</f>
         <v>1</v>
       </c>
-      <c r="B36" s="146" t="s">
+      <c r="B36" s="138" t="s">
         <v>5</v>
       </c>
-      <c r="C36" s="113">
+      <c r="C36" s="112">
         <f>I34 + 1</f>
         <v>4</v>
       </c>
@@ -3057,13 +3075,13 @@
       </c>
     </row>
     <row r="37" spans="1:9" ht="90" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A37" s="141"/>
-      <c r="B37" s="147"/>
-      <c r="C37" s="74"/>
+      <c r="A37" s="150"/>
+      <c r="B37" s="139"/>
+      <c r="C37" s="73"/>
       <c r="D37" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="E37" s="120"/>
+      <c r="E37" s="119"/>
       <c r="F37" s="69" t="s">
         <v>26</v>
       </c>
@@ -3071,15 +3089,15 @@
       <c r="H37" s="6" t="s">
         <v>50</v>
       </c>
-      <c r="I37" s="129" t="s">
+      <c r="I37" s="128" t="s">
         <v>48</v>
       </c>
     </row>
     <row r="38" spans="1:9" ht="15.75" customHeight="1" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="A38" s="142" t="s">
+      <c r="A38" s="155" t="s">
         <v>24</v>
       </c>
-      <c r="B38" s="147"/>
+      <c r="B38" s="139"/>
       <c r="C38" s="18">
         <f>I36 + 1</f>
         <v>11</v>
@@ -3110,9 +3128,9 @@
       </c>
     </row>
     <row r="39" spans="1:9" ht="103.9" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A39" s="143"/>
-      <c r="B39" s="148"/>
-      <c r="C39" s="92"/>
+      <c r="A39" s="156"/>
+      <c r="B39" s="140"/>
+      <c r="C39" s="91"/>
       <c r="D39" s="20" t="s">
         <v>51</v>
       </c>
@@ -3120,7 +3138,7 @@
       <c r="F39" s="20" t="s">
         <v>52</v>
       </c>
-      <c r="G39" s="83" t="s">
+      <c r="G39" s="82" t="s">
         <v>49</v>
       </c>
       <c r="H39" s="59"/>
@@ -3129,6 +3147,17 @@
     <row r="40" spans="1:9" ht="15.75" thickTop="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <mergeCells count="22">
+    <mergeCell ref="A34:A35"/>
+    <mergeCell ref="A36:A37"/>
+    <mergeCell ref="A38:A39"/>
+    <mergeCell ref="B34:B35"/>
+    <mergeCell ref="B36:B39"/>
+    <mergeCell ref="A1:I1"/>
+    <mergeCell ref="A3:A4"/>
+    <mergeCell ref="A5:A6"/>
+    <mergeCell ref="A7:A8"/>
+    <mergeCell ref="A9:A10"/>
+    <mergeCell ref="B3:B4"/>
     <mergeCell ref="B13:B16"/>
     <mergeCell ref="B22:B25"/>
     <mergeCell ref="B28:B33"/>
@@ -3140,17 +3169,6 @@
     <mergeCell ref="A28:A29"/>
     <mergeCell ref="A30:A31"/>
     <mergeCell ref="A32:A33"/>
-    <mergeCell ref="A1:I1"/>
-    <mergeCell ref="A3:A4"/>
-    <mergeCell ref="A5:A6"/>
-    <mergeCell ref="A7:A8"/>
-    <mergeCell ref="A9:A10"/>
-    <mergeCell ref="B3:B4"/>
-    <mergeCell ref="A34:A35"/>
-    <mergeCell ref="A36:A37"/>
-    <mergeCell ref="A38:A39"/>
-    <mergeCell ref="B34:B35"/>
-    <mergeCell ref="B36:B39"/>
   </mergeCells>
   <printOptions horizontalCentered="1" verticalCentered="1"/>
   <pageMargins left="0.25" right="0.25" top="0.25" bottom="0.25" header="0" footer="0"/>

</xml_diff>

<commit_message>
updated schedule for Assign05 due date
</commit_message>
<xml_diff>
--- a/CS320-Spring2025Calendar.xlsx
+++ b/CS320-Spring2025Calendar.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="28429"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="28526"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\cygwin64\home\donha\cs320-spring2025\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1F25D98C-6C5D-4CA2-9B6D-70FB39CEC632}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0EE855FA-C6AF-4E30-A10D-D761871CBDDC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="345" yWindow="570" windowWidth="24345" windowHeight="14730" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Calendar-Sp24" sheetId="1" r:id="rId1"/>
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="88" uniqueCount="83">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="89" uniqueCount="84">
   <si>
     <t>Monday</t>
   </si>
@@ -221,9 +221,6 @@
   <si>
     <t>Team Session: Final Preparation for Milestone 1
 (in-class)</t>
-  </si>
-  <si>
-    <t>Assign06: Team Problem Domain Analysis Submission Review</t>
   </si>
   <si>
     <t>A03: Team MS2
@@ -569,7 +566,17 @@
   </si>
   <si>
     <t>CS320: SW Engineering - Spring 2025 Schedule
-(as of 2-26-2025, subject to change)</t>
+(as of 3-10-2025, subject to change)</t>
+  </si>
+  <si>
+    <t>Team Session:
+Team Analysis &amp; Design Model
+How to Develop a  UML Diagram</t>
+  </si>
+  <si>
+    <t>Team Session:
+Team Analysis &amp; Design Model
+Team Session</t>
   </si>
 </sst>
 </file>
@@ -1489,9 +1496,6 @@
     <xf numFmtId="0" fontId="5" fillId="6" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="6" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1609,9 +1613,6 @@
     <xf numFmtId="0" fontId="5" fillId="3" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="7" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1644,6 +1645,30 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="6" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
@@ -1654,53 +1679,35 @@
     <xf numFmtId="0" fontId="2" fillId="2" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -2029,17 +2036,17 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:17" ht="53.1" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="143" t="s">
-        <v>82</v>
-      </c>
-      <c r="B1" s="144"/>
-      <c r="C1" s="144"/>
-      <c r="D1" s="144"/>
-      <c r="E1" s="144"/>
-      <c r="F1" s="144"/>
-      <c r="G1" s="144"/>
-      <c r="H1" s="144"/>
-      <c r="I1" s="145"/>
+      <c r="A1" s="147" t="s">
+        <v>81</v>
+      </c>
+      <c r="B1" s="148"/>
+      <c r="C1" s="148"/>
+      <c r="D1" s="148"/>
+      <c r="E1" s="148"/>
+      <c r="F1" s="148"/>
+      <c r="G1" s="148"/>
+      <c r="H1" s="148"/>
+      <c r="I1" s="149"/>
     </row>
     <row r="2" spans="1:17" s="2" customFormat="1" ht="21" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
@@ -2061,7 +2068,7 @@
       <c r="G2" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="H2" s="96" t="s">
+      <c r="H2" s="95" t="s">
         <v>4</v>
       </c>
       <c r="I2" s="1" t="s">
@@ -2069,11 +2076,11 @@
       </c>
     </row>
     <row r="3" spans="1:17" ht="15.75" customHeight="1" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="154">
+      <c r="A3" s="138">
         <v>15</v>
       </c>
-      <c r="B3" s="138" t="s">
-        <v>54</v>
+      <c r="B3" s="144" t="s">
+        <v>53</v>
       </c>
       <c r="C3" s="52">
         <v>26</v>
@@ -2094,45 +2101,45 @@
         <f t="shared" si="0"/>
         <v>30</v>
       </c>
-      <c r="H3" s="97">
+      <c r="H3" s="96">
         <f t="shared" si="0"/>
         <v>31</v>
       </c>
-      <c r="I3" s="98">
+      <c r="I3" s="97">
         <f>IF(H3 = 31, 1, H3+1)</f>
         <v>1</v>
       </c>
     </row>
     <row r="4" spans="1:17" ht="101.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="150"/>
-      <c r="B4" s="140"/>
-      <c r="C4" s="99" t="s">
+      <c r="A4" s="139"/>
+      <c r="B4" s="146"/>
+      <c r="C4" s="98" t="s">
         <v>7</v>
       </c>
-      <c r="D4" s="94" t="s">
-        <v>55</v>
+      <c r="D4" s="93" t="s">
+        <v>54</v>
       </c>
       <c r="E4" s="85" t="s">
-        <v>65</v>
-      </c>
-      <c r="F4" s="122" t="s">
-        <v>57</v>
+        <v>64</v>
+      </c>
+      <c r="F4" s="121" t="s">
+        <v>56</v>
       </c>
       <c r="G4" s="32"/>
-      <c r="H4" s="115" t="s">
-        <v>74</v>
-      </c>
-      <c r="I4" s="101"/>
+      <c r="H4" s="114" t="s">
+        <v>73</v>
+      </c>
+      <c r="I4" s="100"/>
     </row>
     <row r="5" spans="1:17" ht="15" customHeight="1" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="153">
+      <c r="A5" s="150">
         <f>A3 - 1</f>
         <v>14</v>
       </c>
-      <c r="B5" s="141" t="s">
+      <c r="B5" s="151" t="s">
         <v>10</v>
       </c>
-      <c r="C5" s="100">
+      <c r="C5" s="99">
         <f>I3 + 1</f>
         <v>2</v>
       </c>
@@ -2162,28 +2169,28 @@
       </c>
     </row>
     <row r="6" spans="1:17" ht="122.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="148"/>
+      <c r="A6" s="137"/>
       <c r="B6" s="142"/>
-      <c r="C6" s="123"/>
+      <c r="C6" s="122"/>
       <c r="D6" s="38" t="s">
+        <v>76</v>
+      </c>
+      <c r="E6" s="39" t="s">
+        <v>74</v>
+      </c>
+      <c r="F6" s="38" t="s">
         <v>77</v>
       </c>
-      <c r="E6" s="39" t="s">
+      <c r="G6" s="39" t="s">
         <v>75</v>
       </c>
-      <c r="F6" s="38" t="s">
-        <v>78</v>
-      </c>
-      <c r="G6" s="39" t="s">
-        <v>76</v>
-      </c>
       <c r="H6" s="38" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="I6" s="70"/>
     </row>
     <row r="7" spans="1:17" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="147">
+      <c r="A7" s="136">
         <f>A5 - 1</f>
         <v>13</v>
       </c>
@@ -2218,26 +2225,26 @@
       </c>
     </row>
     <row r="8" spans="1:17" ht="123.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="147"/>
+      <c r="A8" s="136"/>
       <c r="B8" s="142"/>
-      <c r="C8" s="132" t="s">
+      <c r="C8" s="130" t="s">
         <v>31</v>
       </c>
       <c r="D8" s="38" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="E8" s="61"/>
       <c r="F8" s="11" t="s">
+        <v>78</v>
+      </c>
+      <c r="G8" s="24"/>
+      <c r="H8" s="135" t="s">
         <v>79</v>
       </c>
-      <c r="G8" s="24"/>
-      <c r="H8" s="137" t="s">
-        <v>80</v>
-      </c>
       <c r="I8" s="80"/>
     </row>
     <row r="9" spans="1:17" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="147">
+      <c r="A9" s="136">
         <f>A7 - 1</f>
         <v>12</v>
       </c>
@@ -2279,24 +2286,24 @@
       <c r="Q9" s="74"/>
     </row>
     <row r="10" spans="1:17" ht="102.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="147"/>
+      <c r="A10" s="136"/>
       <c r="B10" s="142"/>
       <c r="C10" s="71" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="D10" s="9" t="s">
         <v>37</v>
       </c>
       <c r="E10" s="61"/>
       <c r="F10" s="9" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="G10" s="10"/>
       <c r="H10" s="9" t="s">
         <v>27</v>
       </c>
-      <c r="I10" s="134" t="s">
-        <v>73</v>
+      <c r="I10" s="132" t="s">
+        <v>72</v>
       </c>
       <c r="K10" s="22"/>
       <c r="L10" s="74"/>
@@ -2307,12 +2314,12 @@
       <c r="Q10" s="75"/>
     </row>
     <row r="11" spans="1:17" ht="15" customHeight="1" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="147">
+      <c r="A11" s="136">
         <f>A9 -1</f>
         <v>11</v>
       </c>
-      <c r="B11" s="141" t="s">
-        <v>56</v>
+      <c r="B11" s="151" t="s">
+        <v>55</v>
       </c>
       <c r="C11" s="15">
         <f>I9 + 1</f>
@@ -2334,11 +2341,11 @@
         <f t="shared" si="1"/>
         <v>27</v>
       </c>
-      <c r="H11" s="102">
+      <c r="H11" s="101">
         <f t="shared" si="1"/>
         <v>28</v>
       </c>
-      <c r="I11" s="108">
+      <c r="I11" s="107">
         <f>IF(H11 = 28,1,H11+1)</f>
         <v>1</v>
       </c>
@@ -2351,21 +2358,21 @@
       <c r="Q11" s="74"/>
     </row>
     <row r="12" spans="1:17" ht="120" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="148"/>
-      <c r="B12" s="146"/>
-      <c r="C12" s="133"/>
+      <c r="A12" s="137"/>
+      <c r="B12" s="143"/>
+      <c r="C12" s="131"/>
       <c r="D12" s="36" t="s">
         <v>41</v>
       </c>
-      <c r="E12" s="124"/>
-      <c r="F12" s="125" t="s">
+      <c r="E12" s="123"/>
+      <c r="F12" s="124" t="s">
         <v>40</v>
       </c>
       <c r="G12" s="34"/>
-      <c r="H12" s="136" t="s">
+      <c r="H12" s="134" t="s">
         <v>21</v>
       </c>
-      <c r="I12" s="109"/>
+      <c r="I12" s="108"/>
       <c r="K12" s="22"/>
       <c r="L12" s="74"/>
       <c r="M12" s="74"/>
@@ -2375,14 +2382,14 @@
       <c r="Q12" s="75"/>
     </row>
     <row r="13" spans="1:17" ht="15" customHeight="1" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="105">
+      <c r="A13" s="104">
         <f xml:space="preserve"> A11 - 1</f>
         <v>10</v>
       </c>
-      <c r="B13" s="138" t="s">
+      <c r="B13" s="144" t="s">
         <v>11</v>
       </c>
-      <c r="C13" s="106">
+      <c r="C13" s="105">
         <f>IF(I11=28, 1, I11+1)</f>
         <v>2</v>
       </c>
@@ -2419,23 +2426,23 @@
       <c r="Q13" s="76"/>
     </row>
     <row r="14" spans="1:17" ht="144.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="104"/>
-      <c r="B14" s="139"/>
+      <c r="A14" s="103"/>
+      <c r="B14" s="145"/>
       <c r="C14" s="83" t="s">
         <v>38</v>
       </c>
       <c r="D14" s="81" t="s">
-        <v>67</v>
-      </c>
-      <c r="E14" s="107"/>
+        <v>66</v>
+      </c>
+      <c r="E14" s="106"/>
       <c r="F14" s="6" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="G14" s="51" t="s">
         <v>28</v>
       </c>
       <c r="H14" s="38" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="I14" s="63" t="s">
         <v>28</v>
@@ -2449,11 +2456,11 @@
       <c r="Q14" s="76"/>
     </row>
     <row r="15" spans="1:17" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="89">
+      <c r="A15" s="88">
         <f>A13 - 1</f>
         <v>9</v>
       </c>
-      <c r="B15" s="139"/>
+      <c r="B15" s="145"/>
       <c r="C15" s="54">
         <f>I13 + 1</f>
         <v>9</v>
@@ -2470,7 +2477,7 @@
         <f t="shared" si="3"/>
         <v>12</v>
       </c>
-      <c r="G15" s="103">
+      <c r="G15" s="102">
         <f t="shared" si="3"/>
         <v>13</v>
       </c>
@@ -2484,33 +2491,28 @@
       </c>
     </row>
     <row r="16" spans="1:17" ht="84" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A16" s="90"/>
-      <c r="B16" s="140"/>
+      <c r="A16" s="89"/>
+      <c r="B16" s="146"/>
       <c r="C16" s="64" t="s">
         <v>28</v>
       </c>
-      <c r="D16" s="8" t="str">
-        <f>F14</f>
+      <c r="D16" s="8" t="s">
+        <v>82</v>
+      </c>
+      <c r="E16" s="50" t="s">
+        <v>25</v>
+      </c>
+      <c r="F16" s="8" t="s">
+        <v>83</v>
+      </c>
+      <c r="G16" s="155"/>
+      <c r="H16" s="50" t="str">
+        <f>F16</f>
         <v>Team Session:
 Team Analysis &amp; Design Model
-Team Git Set-Up</v>
-      </c>
-      <c r="E16" s="50" t="s">
-        <v>25</v>
-      </c>
-      <c r="F16" s="8" t="str">
-        <f>D16</f>
-        <v>Team Session:
-Team Analysis &amp; Design Model
-Team Git Set-Up</v>
-      </c>
-      <c r="G16" s="126" t="s">
-        <v>39</v>
-      </c>
-      <c r="H16" s="50" t="s">
-        <v>43</v>
-      </c>
-      <c r="I16" s="131"/>
+Team Session</v>
+      </c>
+      <c r="I16" s="129"/>
     </row>
     <row r="17" spans="1:17" ht="6.4" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B17" s="21"/>
@@ -2542,8 +2544,8 @@
       <c r="H18" s="29" t="s">
         <v>16</v>
       </c>
-      <c r="I18" s="130" t="s">
-        <v>63</v>
+      <c r="I18" s="128" t="s">
+        <v>62</v>
       </c>
     </row>
     <row r="19" spans="1:17" ht="34.5" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -2557,19 +2559,19 @@
       <c r="I19" s="76"/>
     </row>
     <row r="20" spans="1:17" ht="54" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A20" s="143" t="str">
+      <c r="A20" s="147" t="str">
         <f>A1</f>
         <v>CS320: SW Engineering - Spring 2025 Schedule
-(as of 2-26-2025, subject to change)</v>
-      </c>
-      <c r="B20" s="144"/>
-      <c r="C20" s="144"/>
-      <c r="D20" s="144"/>
-      <c r="E20" s="144"/>
-      <c r="F20" s="144"/>
-      <c r="G20" s="144"/>
-      <c r="H20" s="144"/>
-      <c r="I20" s="145"/>
+(as of 3-10-2025, subject to change)</v>
+      </c>
+      <c r="B20" s="148"/>
+      <c r="C20" s="148"/>
+      <c r="D20" s="148"/>
+      <c r="E20" s="148"/>
+      <c r="F20" s="148"/>
+      <c r="G20" s="148"/>
+      <c r="H20" s="148"/>
+      <c r="I20" s="149"/>
     </row>
     <row r="21" spans="1:17" s="2" customFormat="1" ht="17.25" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A21" s="1" t="str">
@@ -2607,11 +2609,11 @@
       </c>
     </row>
     <row r="22" spans="1:17" ht="15.75" customHeight="1" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="88">
+      <c r="A22" s="87">
         <f>A15-1</f>
         <v>8</v>
       </c>
-      <c r="B22" s="138" t="s">
+      <c r="B22" s="144" t="s">
         <v>11</v>
       </c>
       <c r="C22" s="67">
@@ -2650,10 +2652,12 @@
       <c r="P22" s="74"/>
       <c r="Q22" s="74"/>
     </row>
-    <row r="23" spans="1:17" ht="59.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="89"/>
-      <c r="B23" s="139"/>
-      <c r="C23" s="86"/>
+    <row r="23" spans="1:17" ht="81.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A23" s="88"/>
+      <c r="B23" s="145"/>
+      <c r="C23" s="156" t="s">
+        <v>39</v>
+      </c>
       <c r="D23" s="6" t="s">
         <v>42</v>
       </c>
@@ -2677,11 +2681,11 @@
       <c r="Q23" s="22"/>
     </row>
     <row r="24" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="89">
+      <c r="A24" s="88">
         <f>A22 - 1</f>
         <v>7</v>
       </c>
-      <c r="B24" s="139"/>
+      <c r="B24" s="145"/>
       <c r="C24" s="7">
         <f>I22 + 1</f>
         <v>23</v>
@@ -2719,19 +2723,19 @@
       <c r="Q24" s="74"/>
     </row>
     <row r="25" spans="1:17" ht="129.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A25" s="89"/>
-      <c r="B25" s="139"/>
+      <c r="A25" s="88"/>
+      <c r="B25" s="145"/>
       <c r="C25" s="73"/>
       <c r="D25" s="23" t="s">
         <v>22</v>
       </c>
-      <c r="E25" s="111"/>
-      <c r="F25" s="94" t="s">
+      <c r="E25" s="110"/>
+      <c r="F25" s="93" t="s">
         <v>32</v>
       </c>
-      <c r="G25" s="111"/>
-      <c r="H25" s="87" t="s">
-        <v>70</v>
+      <c r="G25" s="110"/>
+      <c r="H25" s="86" t="s">
+        <v>69</v>
       </c>
       <c r="I25" s="84"/>
       <c r="K25" s="22"/>
@@ -2743,20 +2747,20 @@
       <c r="Q25" s="22"/>
     </row>
     <row r="26" spans="1:17" ht="15" customHeight="1" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="149">
+      <c r="A26" s="152">
         <f>A24 - 1</f>
         <v>6</v>
       </c>
-      <c r="B26" s="92"/>
+      <c r="B26" s="91"/>
       <c r="C26" s="7">
         <f>I24 + 1</f>
         <v>30</v>
       </c>
-      <c r="D26" s="110">
+      <c r="D26" s="109">
         <f>C26 + 1</f>
         <v>31</v>
       </c>
-      <c r="E26" s="100">
+      <c r="E26" s="99">
         <f>IF(D26 = 31, 1, D36+1)</f>
         <v>1</v>
       </c>
@@ -2772,7 +2776,7 @@
         <f t="shared" ref="H26" si="8">G26 + 1</f>
         <v>4</v>
       </c>
-      <c r="I26" s="95">
+      <c r="I26" s="94">
         <f t="shared" ref="I26" si="9">H26 + 1</f>
         <v>5</v>
       </c>
@@ -2785,25 +2789,25 @@
       <c r="Q26" s="74"/>
     </row>
     <row r="27" spans="1:17" ht="68.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A27" s="150"/>
-      <c r="B27" s="93" t="s">
-        <v>53</v>
+      <c r="A27" s="139"/>
+      <c r="B27" s="92" t="s">
+        <v>52</v>
       </c>
       <c r="C27" s="48" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="D27" s="78" t="s">
         <v>19</v>
       </c>
-      <c r="E27" s="113"/>
+      <c r="E27" s="112"/>
       <c r="F27" s="11" t="s">
-        <v>62</v>
-      </c>
-      <c r="G27" s="129"/>
-      <c r="H27" s="127" t="s">
-        <v>44</v>
-      </c>
-      <c r="I27" s="128" t="s">
+        <v>61</v>
+      </c>
+      <c r="G27" s="127"/>
+      <c r="H27" s="125" t="s">
+        <v>43</v>
+      </c>
+      <c r="I27" s="126" t="s">
         <v>34</v>
       </c>
       <c r="K27" s="74"/>
@@ -2815,11 +2819,11 @@
       <c r="Q27" s="22"/>
     </row>
     <row r="28" spans="1:17" ht="15" customHeight="1" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="A28" s="151">
+      <c r="A28" s="153">
         <f>A26 -1</f>
         <v>5</v>
       </c>
-      <c r="B28" s="141" t="s">
+      <c r="B28" s="151" t="s">
         <v>12</v>
       </c>
       <c r="C28" s="12">
@@ -2852,26 +2856,26 @@
       </c>
     </row>
     <row r="29" spans="1:17" ht="55.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A29" s="152"/>
+      <c r="A29" s="154"/>
       <c r="B29" s="142"/>
       <c r="C29" s="15"/>
       <c r="D29" s="9" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="E29" s="39" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="F29" s="38" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="G29" s="24"/>
       <c r="H29" s="11" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="I29" s="25"/>
     </row>
     <row r="30" spans="1:17" ht="15.75" customHeight="1" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="A30" s="153">
+      <c r="A30" s="150">
         <f>A28 -1</f>
         <v>4</v>
       </c>
@@ -2906,14 +2910,14 @@
       </c>
     </row>
     <row r="31" spans="1:17" ht="92.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A31" s="147"/>
+      <c r="A31" s="136"/>
       <c r="B31" s="142"/>
       <c r="C31" s="26"/>
       <c r="D31" s="72" t="s">
         <v>23</v>
       </c>
-      <c r="E31" s="135" t="s">
-        <v>69</v>
+      <c r="E31" s="133" t="s">
+        <v>68</v>
       </c>
       <c r="F31" s="23" t="s">
         <v>33</v>
@@ -2922,13 +2926,13 @@
       <c r="H31" s="55" t="s">
         <v>30</v>
       </c>
-      <c r="I31" s="114" t="str">
+      <c r="I31" s="113" t="str">
         <f>H31</f>
         <v>Spring Break</v>
       </c>
     </row>
     <row r="32" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A32" s="147">
+      <c r="A32" s="136">
         <f>A30 -1</f>
         <v>3</v>
       </c>
@@ -2963,28 +2967,28 @@
       </c>
     </row>
     <row r="33" spans="1:9" ht="52.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A33" s="147"/>
+      <c r="A33" s="136"/>
       <c r="B33" s="142"/>
       <c r="C33" s="54" t="str">
         <f>I31</f>
         <v>Spring Break</v>
       </c>
-      <c r="D33" s="121" t="str">
+      <c r="D33" s="120" t="str">
         <f>I31</f>
         <v>Spring Break</v>
       </c>
       <c r="E33" s="10"/>
       <c r="F33" s="36" t="s">
-        <v>45</v>
-      </c>
-      <c r="G33" s="116"/>
+        <v>44</v>
+      </c>
+      <c r="G33" s="115"/>
       <c r="H33" s="36" t="s">
-        <v>64</v>
-      </c>
-      <c r="I33" s="117"/>
+        <v>63</v>
+      </c>
+      <c r="I33" s="116"/>
     </row>
     <row r="34" spans="1:9" ht="15" customHeight="1" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="A34" s="147">
+      <c r="A34" s="136">
         <f>A32 -1</f>
         <v>2</v>
       </c>
@@ -3003,11 +3007,11 @@
         <f t="shared" ref="E34:I36" si="12">D34 + 1</f>
         <v>29</v>
       </c>
-      <c r="F34" s="102">
+      <c r="F34" s="101">
         <f t="shared" si="12"/>
         <v>30</v>
       </c>
-      <c r="G34" s="112">
+      <c r="G34" s="111">
         <f>IF(F34=30, 1, F34+1)</f>
         <v>1</v>
       </c>
@@ -3021,31 +3025,31 @@
       </c>
     </row>
     <row r="35" spans="1:9" ht="58.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A35" s="148"/>
-      <c r="B35" s="146"/>
+      <c r="A35" s="137"/>
+      <c r="B35" s="143"/>
       <c r="C35" s="45"/>
       <c r="D35" s="35" t="s">
         <v>20</v>
       </c>
       <c r="E35" s="34"/>
-      <c r="F35" s="115" t="s">
+      <c r="F35" s="114" t="s">
         <v>6</v>
       </c>
-      <c r="G35" s="118"/>
+      <c r="G35" s="117"/>
       <c r="H35" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="I35" s="120"/>
+      <c r="I35" s="119"/>
     </row>
     <row r="36" spans="1:9" ht="15" customHeight="1" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="A36" s="154">
+      <c r="A36" s="138">
         <f>A34 -1</f>
         <v>1</v>
       </c>
-      <c r="B36" s="138" t="s">
+      <c r="B36" s="144" t="s">
         <v>5</v>
       </c>
-      <c r="C36" s="112">
+      <c r="C36" s="111">
         <f>I34 + 1</f>
         <v>4</v>
       </c>
@@ -3075,29 +3079,29 @@
       </c>
     </row>
     <row r="37" spans="1:9" ht="90" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A37" s="150"/>
-      <c r="B37" s="139"/>
+      <c r="A37" s="139"/>
+      <c r="B37" s="145"/>
       <c r="C37" s="73"/>
       <c r="D37" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="E37" s="119"/>
+      <c r="E37" s="118"/>
       <c r="F37" s="69" t="s">
         <v>26</v>
       </c>
       <c r="G37" s="6"/>
       <c r="H37" s="6" t="s">
-        <v>50</v>
-      </c>
-      <c r="I37" s="128" t="s">
-        <v>48</v>
+        <v>49</v>
+      </c>
+      <c r="I37" s="126" t="s">
+        <v>47</v>
       </c>
     </row>
     <row r="38" spans="1:9" ht="15.75" customHeight="1" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="A38" s="155" t="s">
+      <c r="A38" s="140" t="s">
         <v>24</v>
       </c>
-      <c r="B38" s="139"/>
+      <c r="B38" s="145"/>
       <c r="C38" s="18">
         <f>I36 + 1</f>
         <v>11</v>
@@ -3128,18 +3132,18 @@
       </c>
     </row>
     <row r="39" spans="1:9" ht="103.9" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A39" s="156"/>
-      <c r="B39" s="140"/>
-      <c r="C39" s="91"/>
+      <c r="A39" s="141"/>
+      <c r="B39" s="146"/>
+      <c r="C39" s="90"/>
       <c r="D39" s="20" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="E39" s="49"/>
       <c r="F39" s="20" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="G39" s="82" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="H39" s="59"/>
       <c r="I39" s="60"/>
@@ -3147,17 +3151,6 @@
     <row r="40" spans="1:9" ht="15.75" thickTop="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <mergeCells count="22">
-    <mergeCell ref="A34:A35"/>
-    <mergeCell ref="A36:A37"/>
-    <mergeCell ref="A38:A39"/>
-    <mergeCell ref="B34:B35"/>
-    <mergeCell ref="B36:B39"/>
-    <mergeCell ref="A1:I1"/>
-    <mergeCell ref="A3:A4"/>
-    <mergeCell ref="A5:A6"/>
-    <mergeCell ref="A7:A8"/>
-    <mergeCell ref="A9:A10"/>
-    <mergeCell ref="B3:B4"/>
     <mergeCell ref="B13:B16"/>
     <mergeCell ref="B22:B25"/>
     <mergeCell ref="B28:B33"/>
@@ -3169,6 +3162,17 @@
     <mergeCell ref="A28:A29"/>
     <mergeCell ref="A30:A31"/>
     <mergeCell ref="A32:A33"/>
+    <mergeCell ref="A1:I1"/>
+    <mergeCell ref="A3:A4"/>
+    <mergeCell ref="A5:A6"/>
+    <mergeCell ref="A7:A8"/>
+    <mergeCell ref="A9:A10"/>
+    <mergeCell ref="B3:B4"/>
+    <mergeCell ref="A34:A35"/>
+    <mergeCell ref="A36:A37"/>
+    <mergeCell ref="A38:A39"/>
+    <mergeCell ref="B34:B35"/>
+    <mergeCell ref="B36:B39"/>
   </mergeCells>
   <printOptions horizontalCentered="1" verticalCentered="1"/>
   <pageMargins left="0.25" right="0.25" top="0.25" bottom="0.25" header="0" footer="0"/>

</xml_diff>

<commit_message>
updated midterm evals due date
</commit_message>
<xml_diff>
--- a/CS320-Spring2025Calendar.xlsx
+++ b/CS320-Spring2025Calendar.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\cygwin64\home\donha\cs320-spring2025\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0EE855FA-C6AF-4E30-A10D-D761871CBDDC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D329E5BB-604C-4244-B039-7A3A8042AA45}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="435" yWindow="345" windowWidth="27435" windowHeight="14325" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Calendar-Sp24" sheetId="1" r:id="rId1"/>
@@ -565,10 +565,6 @@
     </r>
   </si>
   <si>
-    <t>CS320: SW Engineering - Spring 2025 Schedule
-(as of 3-10-2025, subject to change)</t>
-  </si>
-  <si>
     <t>Team Session:
 Team Analysis &amp; Design Model
 How to Develop a  UML Diagram</t>
@@ -577,6 +573,10 @@
     <t>Team Session:
 Team Analysis &amp; Design Model
 Team Session</t>
+  </si>
+  <si>
+    <t>CS320: SW Engineering - Spring 2025 Schedule
+(as of 3-18-2025, subject to change)</t>
   </si>
 </sst>
 </file>
@@ -1239,7 +1239,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="157">
+  <cellXfs count="159">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -1646,16 +1646,58 @@
     <xf numFmtId="0" fontId="3" fillId="6" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1664,49 +1706,13 @@
     <xf numFmtId="0" fontId="9" fillId="2" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -2036,17 +2042,17 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:17" ht="53.1" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="147" t="s">
-        <v>81</v>
-      </c>
-      <c r="B1" s="148"/>
-      <c r="C1" s="148"/>
-      <c r="D1" s="148"/>
-      <c r="E1" s="148"/>
-      <c r="F1" s="148"/>
-      <c r="G1" s="148"/>
-      <c r="H1" s="148"/>
-      <c r="I1" s="149"/>
+      <c r="A1" s="142" t="s">
+        <v>83</v>
+      </c>
+      <c r="B1" s="143"/>
+      <c r="C1" s="143"/>
+      <c r="D1" s="143"/>
+      <c r="E1" s="143"/>
+      <c r="F1" s="143"/>
+      <c r="G1" s="143"/>
+      <c r="H1" s="143"/>
+      <c r="I1" s="144"/>
     </row>
     <row r="2" spans="1:17" s="2" customFormat="1" ht="21" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
@@ -2076,10 +2082,10 @@
       </c>
     </row>
     <row r="3" spans="1:17" ht="15.75" customHeight="1" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="138">
+      <c r="A3" s="153">
         <v>15</v>
       </c>
-      <c r="B3" s="144" t="s">
+      <c r="B3" s="137" t="s">
         <v>53</v>
       </c>
       <c r="C3" s="52">
@@ -2111,8 +2117,8 @@
       </c>
     </row>
     <row r="4" spans="1:17" ht="101.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="139"/>
-      <c r="B4" s="146"/>
+      <c r="A4" s="149"/>
+      <c r="B4" s="139"/>
       <c r="C4" s="98" t="s">
         <v>7</v>
       </c>
@@ -2132,11 +2138,11 @@
       <c r="I4" s="100"/>
     </row>
     <row r="5" spans="1:17" ht="15" customHeight="1" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="150">
+      <c r="A5" s="152">
         <f>A3 - 1</f>
         <v>14</v>
       </c>
-      <c r="B5" s="151" t="s">
+      <c r="B5" s="140" t="s">
         <v>10</v>
       </c>
       <c r="C5" s="99">
@@ -2169,8 +2175,8 @@
       </c>
     </row>
     <row r="6" spans="1:17" ht="122.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="137"/>
-      <c r="B6" s="142"/>
+      <c r="A6" s="147"/>
+      <c r="B6" s="141"/>
       <c r="C6" s="122"/>
       <c r="D6" s="38" t="s">
         <v>76</v>
@@ -2190,11 +2196,11 @@
       <c r="I6" s="70"/>
     </row>
     <row r="7" spans="1:17" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="136">
+      <c r="A7" s="146">
         <f>A5 - 1</f>
         <v>13</v>
       </c>
-      <c r="B7" s="142"/>
+      <c r="B7" s="141"/>
       <c r="C7" s="15">
         <f>I5 + 1</f>
         <v>9</v>
@@ -2225,8 +2231,8 @@
       </c>
     </row>
     <row r="8" spans="1:17" ht="123.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="136"/>
-      <c r="B8" s="142"/>
+      <c r="A8" s="146"/>
+      <c r="B8" s="141"/>
       <c r="C8" s="130" t="s">
         <v>31</v>
       </c>
@@ -2244,11 +2250,11 @@
       <c r="I8" s="80"/>
     </row>
     <row r="9" spans="1:17" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="136">
+      <c r="A9" s="146">
         <f>A7 - 1</f>
         <v>12</v>
       </c>
-      <c r="B9" s="142"/>
+      <c r="B9" s="141"/>
       <c r="C9" s="12">
         <f>I7 + 1</f>
         <v>16</v>
@@ -2286,8 +2292,8 @@
       <c r="Q9" s="74"/>
     </row>
     <row r="10" spans="1:17" ht="102.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="136"/>
-      <c r="B10" s="142"/>
+      <c r="A10" s="146"/>
+      <c r="B10" s="141"/>
       <c r="C10" s="71" t="s">
         <v>67</v>
       </c>
@@ -2314,11 +2320,11 @@
       <c r="Q10" s="75"/>
     </row>
     <row r="11" spans="1:17" ht="15" customHeight="1" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="136">
+      <c r="A11" s="146">
         <f>A9 -1</f>
         <v>11</v>
       </c>
-      <c r="B11" s="151" t="s">
+      <c r="B11" s="140" t="s">
         <v>55</v>
       </c>
       <c r="C11" s="15">
@@ -2358,8 +2364,8 @@
       <c r="Q11" s="74"/>
     </row>
     <row r="12" spans="1:17" ht="120" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="137"/>
-      <c r="B12" s="143"/>
+      <c r="A12" s="147"/>
+      <c r="B12" s="145"/>
       <c r="C12" s="131"/>
       <c r="D12" s="36" t="s">
         <v>41</v>
@@ -2386,7 +2392,7 @@
         <f xml:space="preserve"> A11 - 1</f>
         <v>10</v>
       </c>
-      <c r="B13" s="144" t="s">
+      <c r="B13" s="137" t="s">
         <v>11</v>
       </c>
       <c r="C13" s="105">
@@ -2427,7 +2433,7 @@
     </row>
     <row r="14" spans="1:17" ht="144.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="103"/>
-      <c r="B14" s="145"/>
+      <c r="B14" s="138"/>
       <c r="C14" s="83" t="s">
         <v>38</v>
       </c>
@@ -2460,7 +2466,7 @@
         <f>A13 - 1</f>
         <v>9</v>
       </c>
-      <c r="B15" s="145"/>
+      <c r="B15" s="138"/>
       <c r="C15" s="54">
         <f>I13 + 1</f>
         <v>9</v>
@@ -2492,20 +2498,20 @@
     </row>
     <row r="16" spans="1:17" ht="84" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A16" s="89"/>
-      <c r="B16" s="146"/>
+      <c r="B16" s="139"/>
       <c r="C16" s="64" t="s">
         <v>28</v>
       </c>
       <c r="D16" s="8" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="E16" s="50" t="s">
         <v>25</v>
       </c>
       <c r="F16" s="8" t="s">
-        <v>83</v>
-      </c>
-      <c r="G16" s="155"/>
+        <v>82</v>
+      </c>
+      <c r="G16" s="136"/>
       <c r="H16" s="50" t="str">
         <f>F16</f>
         <v>Team Session:
@@ -2559,19 +2565,19 @@
       <c r="I19" s="76"/>
     </row>
     <row r="20" spans="1:17" ht="54" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A20" s="147" t="str">
+      <c r="A20" s="142" t="str">
         <f>A1</f>
         <v>CS320: SW Engineering - Spring 2025 Schedule
-(as of 3-10-2025, subject to change)</v>
-      </c>
-      <c r="B20" s="148"/>
-      <c r="C20" s="148"/>
-      <c r="D20" s="148"/>
-      <c r="E20" s="148"/>
-      <c r="F20" s="148"/>
-      <c r="G20" s="148"/>
-      <c r="H20" s="148"/>
-      <c r="I20" s="149"/>
+(as of 3-18-2025, subject to change)</v>
+      </c>
+      <c r="B20" s="143"/>
+      <c r="C20" s="143"/>
+      <c r="D20" s="143"/>
+      <c r="E20" s="143"/>
+      <c r="F20" s="143"/>
+      <c r="G20" s="143"/>
+      <c r="H20" s="143"/>
+      <c r="I20" s="144"/>
     </row>
     <row r="21" spans="1:17" s="2" customFormat="1" ht="17.25" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A21" s="1" t="str">
@@ -2613,7 +2619,7 @@
         <f>A15-1</f>
         <v>8</v>
       </c>
-      <c r="B22" s="144" t="s">
+      <c r="B22" s="137" t="s">
         <v>11</v>
       </c>
       <c r="C22" s="67">
@@ -2654,8 +2660,8 @@
     </row>
     <row r="23" spans="1:17" ht="81.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="88"/>
-      <c r="B23" s="145"/>
-      <c r="C23" s="156" t="s">
+      <c r="B23" s="138"/>
+      <c r="C23" s="158" t="s">
         <v>39</v>
       </c>
       <c r="D23" s="6" t="s">
@@ -2685,7 +2691,7 @@
         <f>A22 - 1</f>
         <v>7</v>
       </c>
-      <c r="B24" s="145"/>
+      <c r="B24" s="138"/>
       <c r="C24" s="7">
         <f>I22 + 1</f>
         <v>23</v>
@@ -2724,12 +2730,14 @@
     </row>
     <row r="25" spans="1:17" ht="129.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A25" s="88"/>
-      <c r="B25" s="145"/>
+      <c r="B25" s="138"/>
       <c r="C25" s="73"/>
       <c r="D25" s="23" t="s">
         <v>22</v>
       </c>
-      <c r="E25" s="110"/>
+      <c r="E25" s="156" t="s">
+        <v>34</v>
+      </c>
       <c r="F25" s="93" t="s">
         <v>32</v>
       </c>
@@ -2747,7 +2755,7 @@
       <c r="Q25" s="22"/>
     </row>
     <row r="26" spans="1:17" ht="15" customHeight="1" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="152">
+      <c r="A26" s="148">
         <f>A24 - 1</f>
         <v>6</v>
       </c>
@@ -2789,7 +2797,7 @@
       <c r="Q26" s="74"/>
     </row>
     <row r="27" spans="1:17" ht="68.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A27" s="139"/>
+      <c r="A27" s="149"/>
       <c r="B27" s="92" t="s">
         <v>52</v>
       </c>
@@ -2807,9 +2815,7 @@
       <c r="H27" s="125" t="s">
         <v>43</v>
       </c>
-      <c r="I27" s="126" t="s">
-        <v>34</v>
-      </c>
+      <c r="I27" s="157"/>
       <c r="K27" s="74"/>
       <c r="L27" s="74"/>
       <c r="M27" s="22"/>
@@ -2819,11 +2825,11 @@
       <c r="Q27" s="22"/>
     </row>
     <row r="28" spans="1:17" ht="15" customHeight="1" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="A28" s="153">
+      <c r="A28" s="150">
         <f>A26 -1</f>
         <v>5</v>
       </c>
-      <c r="B28" s="151" t="s">
+      <c r="B28" s="140" t="s">
         <v>12</v>
       </c>
       <c r="C28" s="12">
@@ -2856,8 +2862,8 @@
       </c>
     </row>
     <row r="29" spans="1:17" ht="55.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A29" s="154"/>
-      <c r="B29" s="142"/>
+      <c r="A29" s="151"/>
+      <c r="B29" s="141"/>
       <c r="C29" s="15"/>
       <c r="D29" s="9" t="s">
         <v>65</v>
@@ -2875,11 +2881,11 @@
       <c r="I29" s="25"/>
     </row>
     <row r="30" spans="1:17" ht="15.75" customHeight="1" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="A30" s="150">
+      <c r="A30" s="152">
         <f>A28 -1</f>
         <v>4</v>
       </c>
-      <c r="B30" s="142"/>
+      <c r="B30" s="141"/>
       <c r="C30" s="47">
         <f>I28 + 1</f>
         <v>13</v>
@@ -2910,8 +2916,8 @@
       </c>
     </row>
     <row r="31" spans="1:17" ht="92.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A31" s="136"/>
-      <c r="B31" s="142"/>
+      <c r="A31" s="146"/>
+      <c r="B31" s="141"/>
       <c r="C31" s="26"/>
       <c r="D31" s="72" t="s">
         <v>23</v>
@@ -2932,11 +2938,11 @@
       </c>
     </row>
     <row r="32" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A32" s="136">
+      <c r="A32" s="146">
         <f>A30 -1</f>
         <v>3</v>
       </c>
-      <c r="B32" s="142"/>
+      <c r="B32" s="141"/>
       <c r="C32" s="24">
         <f>I30 + 1</f>
         <v>20</v>
@@ -2967,8 +2973,8 @@
       </c>
     </row>
     <row r="33" spans="1:9" ht="52.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A33" s="136"/>
-      <c r="B33" s="142"/>
+      <c r="A33" s="146"/>
+      <c r="B33" s="141"/>
       <c r="C33" s="54" t="str">
         <f>I31</f>
         <v>Spring Break</v>
@@ -2988,11 +2994,11 @@
       <c r="I33" s="116"/>
     </row>
     <row r="34" spans="1:9" ht="15" customHeight="1" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="A34" s="136">
+      <c r="A34" s="146">
         <f>A32 -1</f>
         <v>2</v>
       </c>
-      <c r="B34" s="142" t="s">
+      <c r="B34" s="141" t="s">
         <v>29</v>
       </c>
       <c r="C34" s="26">
@@ -3025,8 +3031,8 @@
       </c>
     </row>
     <row r="35" spans="1:9" ht="58.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A35" s="137"/>
-      <c r="B35" s="143"/>
+      <c r="A35" s="147"/>
+      <c r="B35" s="145"/>
       <c r="C35" s="45"/>
       <c r="D35" s="35" t="s">
         <v>20</v>
@@ -3042,11 +3048,11 @@
       <c r="I35" s="119"/>
     </row>
     <row r="36" spans="1:9" ht="15" customHeight="1" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="A36" s="138">
+      <c r="A36" s="153">
         <f>A34 -1</f>
         <v>1</v>
       </c>
-      <c r="B36" s="144" t="s">
+      <c r="B36" s="137" t="s">
         <v>5</v>
       </c>
       <c r="C36" s="111">
@@ -3079,8 +3085,8 @@
       </c>
     </row>
     <row r="37" spans="1:9" ht="90" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A37" s="139"/>
-      <c r="B37" s="145"/>
+      <c r="A37" s="149"/>
+      <c r="B37" s="138"/>
       <c r="C37" s="73"/>
       <c r="D37" s="6" t="s">
         <v>6</v>
@@ -3098,10 +3104,10 @@
       </c>
     </row>
     <row r="38" spans="1:9" ht="15.75" customHeight="1" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="A38" s="140" t="s">
+      <c r="A38" s="154" t="s">
         <v>24</v>
       </c>
-      <c r="B38" s="145"/>
+      <c r="B38" s="138"/>
       <c r="C38" s="18">
         <f>I36 + 1</f>
         <v>11</v>
@@ -3132,8 +3138,8 @@
       </c>
     </row>
     <row r="39" spans="1:9" ht="103.9" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A39" s="141"/>
-      <c r="B39" s="146"/>
+      <c r="A39" s="155"/>
+      <c r="B39" s="139"/>
       <c r="C39" s="90"/>
       <c r="D39" s="20" t="s">
         <v>50</v>
@@ -3151,6 +3157,17 @@
     <row r="40" spans="1:9" ht="15.75" thickTop="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <mergeCells count="22">
+    <mergeCell ref="A34:A35"/>
+    <mergeCell ref="A36:A37"/>
+    <mergeCell ref="A38:A39"/>
+    <mergeCell ref="B34:B35"/>
+    <mergeCell ref="B36:B39"/>
+    <mergeCell ref="A1:I1"/>
+    <mergeCell ref="A3:A4"/>
+    <mergeCell ref="A5:A6"/>
+    <mergeCell ref="A7:A8"/>
+    <mergeCell ref="A9:A10"/>
+    <mergeCell ref="B3:B4"/>
     <mergeCell ref="B13:B16"/>
     <mergeCell ref="B22:B25"/>
     <mergeCell ref="B28:B33"/>
@@ -3162,17 +3179,6 @@
     <mergeCell ref="A28:A29"/>
     <mergeCell ref="A30:A31"/>
     <mergeCell ref="A32:A33"/>
-    <mergeCell ref="A1:I1"/>
-    <mergeCell ref="A3:A4"/>
-    <mergeCell ref="A5:A6"/>
-    <mergeCell ref="A7:A8"/>
-    <mergeCell ref="A9:A10"/>
-    <mergeCell ref="B3:B4"/>
-    <mergeCell ref="A34:A35"/>
-    <mergeCell ref="A36:A37"/>
-    <mergeCell ref="A38:A39"/>
-    <mergeCell ref="B34:B35"/>
-    <mergeCell ref="B36:B39"/>
   </mergeCells>
   <printOptions horizontalCentered="1" verticalCentered="1"/>
   <pageMargins left="0.25" right="0.25" top="0.25" bottom="0.25" header="0" footer="0"/>

</xml_diff>

<commit_message>
updated schedule and calendar
</commit_message>
<xml_diff>
--- a/CS320-Spring2025Calendar.xlsx
+++ b/CS320-Spring2025Calendar.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\cygwin64\home\donha\cs320-spring2025\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D329E5BB-604C-4244-B039-7A3A8042AA45}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EAE2822C-23CF-4D12-9342-FDA2B932AF99}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="435" yWindow="345" windowWidth="27435" windowHeight="14325" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="300" yWindow="285" windowWidth="25290" windowHeight="14325" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Calendar-Sp24" sheetId="1" r:id="rId1"/>
@@ -94,10 +94,6 @@
     <t>Legend</t>
   </si>
   <si>
-    <t>SQL/JDBC/ORM Review &amp; Labs
-(in class)</t>
-  </si>
-  <si>
     <t>A03: Team MS3
 75% Working System
 (w/SQL DB)</t>
@@ -143,25 +139,6 @@
   <si>
     <t>A02: Individual Project Proposal due Noon
 (Marmoset)</t>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">Lecture 13: Relational Databases
-Lecture 14: DB Applications, JDBC
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="9"/>
-        <color rgb="FFFF0000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Lab 4: SQL (assigned)
-Lab05: JDBC (assigned)</t>
-    </r>
   </si>
   <si>
     <t>Library Example Project
@@ -229,9 +206,6 @@
   <si>
     <t>Lecture 16: Testing
 Lecture 17: Quality Assurance</t>
-  </si>
-  <si>
-    <t>DB Testing &amp; General Questions about Lab06</t>
   </si>
   <si>
     <t>ORM Review (Lab06)</t>
@@ -412,27 +386,6 @@
 (Marmoset)</t>
   </si>
   <si>
-    <r>
-      <t xml:space="preserve">Lecture  15: ORM, Designing a Persistence Layer
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="9"/>
-        <color rgb="FFFF0000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Lab 6: ORM
-(assigned)
-Lab 4: SQL
-due by Noon
-(Marmoset)</t>
-    </r>
-  </si>
-  <si>
     <t>Lab 5: JDBC
 due Mon by Noon
 -------------&gt;&gt;&gt;&gt;
@@ -576,7 +529,52 @@
   </si>
   <si>
     <t>CS320: SW Engineering - Spring 2025 Schedule
-(as of 3-18-2025, subject to change)</t>
+(as of 3-29-2025, subject to change)</t>
+  </si>
+  <si>
+    <t>ORM &amp; SQL DB Review and DB Testing</t>
+  </si>
+  <si>
+    <t>Lecture  15: ORM, Designing a Persistence Layer</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Lecture 13: Relational Databases
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="9"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Lab 4: SQL (assigned)
+Lab05: JDBC (assigned)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Lecture 14: DB Applications, JDBC
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="9"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Lab 6: ORM
+(assigned)
+Lab 4: SQL
+due by Noon
+(Marmoset)</t>
+    </r>
   </si>
 </sst>
 </file>
@@ -1239,7 +1237,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="159">
+  <cellXfs count="158">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -1649,6 +1647,36 @@
     <xf numFmtId="0" fontId="5" fillId="2" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
     </xf>
@@ -1658,61 +1686,28 @@
     <xf numFmtId="0" fontId="2" fillId="2" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="6" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -2042,17 +2037,17 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:17" ht="53.1" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="142" t="s">
-        <v>83</v>
-      </c>
-      <c r="B1" s="143"/>
-      <c r="C1" s="143"/>
-      <c r="D1" s="143"/>
-      <c r="E1" s="143"/>
-      <c r="F1" s="143"/>
-      <c r="G1" s="143"/>
-      <c r="H1" s="143"/>
-      <c r="I1" s="144"/>
+      <c r="A1" s="150" t="s">
+        <v>79</v>
+      </c>
+      <c r="B1" s="151"/>
+      <c r="C1" s="151"/>
+      <c r="D1" s="151"/>
+      <c r="E1" s="151"/>
+      <c r="F1" s="151"/>
+      <c r="G1" s="151"/>
+      <c r="H1" s="151"/>
+      <c r="I1" s="152"/>
     </row>
     <row r="2" spans="1:17" s="2" customFormat="1" ht="21" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
@@ -2082,11 +2077,11 @@
       </c>
     </row>
     <row r="3" spans="1:17" ht="15.75" customHeight="1" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="153">
+      <c r="A3" s="141">
         <v>15</v>
       </c>
-      <c r="B3" s="137" t="s">
-        <v>53</v>
+      <c r="B3" s="147" t="s">
+        <v>50</v>
       </c>
       <c r="C3" s="52">
         <v>26</v>
@@ -2117,32 +2112,32 @@
       </c>
     </row>
     <row r="4" spans="1:17" ht="101.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="149"/>
-      <c r="B4" s="139"/>
+      <c r="A4" s="142"/>
+      <c r="B4" s="149"/>
       <c r="C4" s="98" t="s">
         <v>7</v>
       </c>
       <c r="D4" s="93" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="E4" s="85" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="F4" s="121" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="G4" s="32"/>
       <c r="H4" s="114" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="I4" s="100"/>
     </row>
     <row r="5" spans="1:17" ht="15" customHeight="1" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="152">
+      <c r="A5" s="153">
         <f>A3 - 1</f>
         <v>14</v>
       </c>
-      <c r="B5" s="140" t="s">
+      <c r="B5" s="154" t="s">
         <v>10</v>
       </c>
       <c r="C5" s="99">
@@ -2175,32 +2170,32 @@
       </c>
     </row>
     <row r="6" spans="1:17" ht="122.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="147"/>
-      <c r="B6" s="141"/>
+      <c r="A6" s="140"/>
+      <c r="B6" s="145"/>
       <c r="C6" s="122"/>
       <c r="D6" s="38" t="s">
-        <v>76</v>
+        <v>72</v>
       </c>
       <c r="E6" s="39" t="s">
-        <v>74</v>
+        <v>70</v>
       </c>
       <c r="F6" s="38" t="s">
-        <v>77</v>
+        <v>73</v>
       </c>
       <c r="G6" s="39" t="s">
-        <v>75</v>
+        <v>71</v>
       </c>
       <c r="H6" s="38" t="s">
-        <v>57</v>
+        <v>54</v>
       </c>
       <c r="I6" s="70"/>
     </row>
     <row r="7" spans="1:17" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="146">
+      <c r="A7" s="139">
         <f>A5 - 1</f>
         <v>13</v>
       </c>
-      <c r="B7" s="141"/>
+      <c r="B7" s="145"/>
       <c r="C7" s="15">
         <f>I5 + 1</f>
         <v>9</v>
@@ -2231,30 +2226,30 @@
       </c>
     </row>
     <row r="8" spans="1:17" ht="123.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="146"/>
-      <c r="B8" s="141"/>
+      <c r="A8" s="139"/>
+      <c r="B8" s="145"/>
       <c r="C8" s="130" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="D8" s="38" t="s">
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="E8" s="61"/>
       <c r="F8" s="11" t="s">
-        <v>78</v>
+        <v>74</v>
       </c>
       <c r="G8" s="24"/>
       <c r="H8" s="135" t="s">
-        <v>79</v>
+        <v>75</v>
       </c>
       <c r="I8" s="80"/>
     </row>
     <row r="9" spans="1:17" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="146">
+      <c r="A9" s="139">
         <f>A7 - 1</f>
         <v>12</v>
       </c>
-      <c r="B9" s="141"/>
+      <c r="B9" s="145"/>
       <c r="C9" s="12">
         <f>I7 + 1</f>
         <v>16</v>
@@ -2292,24 +2287,24 @@
       <c r="Q9" s="74"/>
     </row>
     <row r="10" spans="1:17" ht="102.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="146"/>
-      <c r="B10" s="141"/>
+      <c r="A10" s="139"/>
+      <c r="B10" s="145"/>
       <c r="C10" s="71" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
       <c r="D10" s="9" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="E10" s="61"/>
       <c r="F10" s="9" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="G10" s="10"/>
       <c r="H10" s="9" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="I10" s="132" t="s">
-        <v>72</v>
+        <v>68</v>
       </c>
       <c r="K10" s="22"/>
       <c r="L10" s="74"/>
@@ -2320,12 +2315,12 @@
       <c r="Q10" s="75"/>
     </row>
     <row r="11" spans="1:17" ht="15" customHeight="1" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="146">
+      <c r="A11" s="139">
         <f>A9 -1</f>
         <v>11</v>
       </c>
-      <c r="B11" s="140" t="s">
-        <v>55</v>
+      <c r="B11" s="154" t="s">
+        <v>52</v>
       </c>
       <c r="C11" s="15">
         <f>I9 + 1</f>
@@ -2364,19 +2359,19 @@
       <c r="Q11" s="74"/>
     </row>
     <row r="12" spans="1:17" ht="120" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="147"/>
-      <c r="B12" s="145"/>
+      <c r="A12" s="140"/>
+      <c r="B12" s="146"/>
       <c r="C12" s="131"/>
       <c r="D12" s="36" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="E12" s="123"/>
       <c r="F12" s="124" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="G12" s="34"/>
       <c r="H12" s="134" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="I12" s="108"/>
       <c r="K12" s="22"/>
@@ -2392,7 +2387,7 @@
         <f xml:space="preserve"> A11 - 1</f>
         <v>10</v>
       </c>
-      <c r="B13" s="137" t="s">
+      <c r="B13" s="147" t="s">
         <v>11</v>
       </c>
       <c r="C13" s="105">
@@ -2433,25 +2428,25 @@
     </row>
     <row r="14" spans="1:17" ht="144.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="103"/>
-      <c r="B14" s="138"/>
+      <c r="B14" s="148"/>
       <c r="C14" s="83" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="D14" s="81" t="s">
-        <v>66</v>
+        <v>63</v>
       </c>
       <c r="E14" s="106"/>
       <c r="F14" s="6" t="s">
-        <v>60</v>
+        <v>57</v>
       </c>
       <c r="G14" s="51" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="H14" s="38" t="s">
-        <v>80</v>
+        <v>76</v>
       </c>
       <c r="I14" s="63" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="K14" s="76"/>
       <c r="L14" s="22"/>
@@ -2466,7 +2461,7 @@
         <f>A13 - 1</f>
         <v>9</v>
       </c>
-      <c r="B15" s="138"/>
+      <c r="B15" s="148"/>
       <c r="C15" s="54">
         <f>I13 + 1</f>
         <v>9</v>
@@ -2498,18 +2493,18 @@
     </row>
     <row r="16" spans="1:17" ht="84" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A16" s="89"/>
-      <c r="B16" s="139"/>
+      <c r="B16" s="149"/>
       <c r="C16" s="64" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="D16" s="8" t="s">
-        <v>81</v>
+        <v>77</v>
       </c>
       <c r="E16" s="50" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="F16" s="8" t="s">
-        <v>82</v>
+        <v>78</v>
       </c>
       <c r="G16" s="136"/>
       <c r="H16" s="50" t="str">
@@ -2539,19 +2534,19 @@
         <v>14</v>
       </c>
       <c r="E18" s="27" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="F18" s="28" t="s">
         <v>15</v>
       </c>
       <c r="G18" s="79" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="H18" s="29" t="s">
         <v>16</v>
       </c>
       <c r="I18" s="128" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
     </row>
     <row r="19" spans="1:17" ht="34.5" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -2565,19 +2560,19 @@
       <c r="I19" s="76"/>
     </row>
     <row r="20" spans="1:17" ht="54" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A20" s="142" t="str">
+      <c r="A20" s="150" t="str">
         <f>A1</f>
         <v>CS320: SW Engineering - Spring 2025 Schedule
-(as of 3-18-2025, subject to change)</v>
-      </c>
-      <c r="B20" s="143"/>
-      <c r="C20" s="143"/>
-      <c r="D20" s="143"/>
-      <c r="E20" s="143"/>
-      <c r="F20" s="143"/>
-      <c r="G20" s="143"/>
-      <c r="H20" s="143"/>
-      <c r="I20" s="144"/>
+(as of 3-29-2025, subject to change)</v>
+      </c>
+      <c r="B20" s="151"/>
+      <c r="C20" s="151"/>
+      <c r="D20" s="151"/>
+      <c r="E20" s="151"/>
+      <c r="F20" s="151"/>
+      <c r="G20" s="151"/>
+      <c r="H20" s="151"/>
+      <c r="I20" s="152"/>
     </row>
     <row r="21" spans="1:17" s="2" customFormat="1" ht="17.25" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A21" s="1" t="str">
@@ -2619,7 +2614,7 @@
         <f>A15-1</f>
         <v>8</v>
       </c>
-      <c r="B22" s="137" t="s">
+      <c r="B22" s="147" t="s">
         <v>11</v>
       </c>
       <c r="C22" s="67">
@@ -2660,12 +2655,12 @@
     </row>
     <row r="23" spans="1:17" ht="81.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="88"/>
-      <c r="B23" s="138"/>
-      <c r="C23" s="158" t="s">
-        <v>39</v>
+      <c r="B23" s="148"/>
+      <c r="C23" s="138" t="s">
+        <v>37</v>
       </c>
       <c r="D23" s="6" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="E23" s="43"/>
       <c r="F23" s="6" t="str">
@@ -2691,7 +2686,7 @@
         <f>A22 - 1</f>
         <v>7</v>
       </c>
-      <c r="B24" s="138"/>
+      <c r="B24" s="148"/>
       <c r="C24" s="7">
         <f>I22 + 1</f>
         <v>23</v>
@@ -2730,20 +2725,20 @@
     </row>
     <row r="25" spans="1:17" ht="129.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A25" s="88"/>
-      <c r="B25" s="138"/>
+      <c r="B25" s="148"/>
       <c r="C25" s="73"/>
       <c r="D25" s="23" t="s">
-        <v>22</v>
-      </c>
-      <c r="E25" s="156" t="s">
-        <v>34</v>
+        <v>21</v>
+      </c>
+      <c r="E25" s="137" t="s">
+        <v>32</v>
       </c>
       <c r="F25" s="93" t="s">
-        <v>32</v>
+        <v>82</v>
       </c>
       <c r="G25" s="110"/>
       <c r="H25" s="86" t="s">
-        <v>69</v>
+        <v>83</v>
       </c>
       <c r="I25" s="84"/>
       <c r="K25" s="22"/>
@@ -2755,7 +2750,7 @@
       <c r="Q25" s="22"/>
     </row>
     <row r="26" spans="1:17" ht="15" customHeight="1" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="148">
+      <c r="A26" s="155">
         <f>A24 - 1</f>
         <v>6</v>
       </c>
@@ -2797,25 +2792,25 @@
       <c r="Q26" s="74"/>
     </row>
     <row r="27" spans="1:17" ht="68.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A27" s="149"/>
+      <c r="A27" s="142"/>
       <c r="B27" s="92" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="C27" s="48" t="s">
-        <v>70</v>
+        <v>66</v>
       </c>
       <c r="D27" s="78" t="s">
-        <v>19</v>
+        <v>81</v>
       </c>
       <c r="E27" s="112"/>
       <c r="F27" s="11" t="s">
-        <v>61</v>
+        <v>58</v>
       </c>
       <c r="G27" s="127"/>
       <c r="H27" s="125" t="s">
-        <v>43</v>
-      </c>
-      <c r="I27" s="157"/>
+        <v>41</v>
+      </c>
+      <c r="I27" s="25"/>
       <c r="K27" s="74"/>
       <c r="L27" s="74"/>
       <c r="M27" s="22"/>
@@ -2825,11 +2820,11 @@
       <c r="Q27" s="22"/>
     </row>
     <row r="28" spans="1:17" ht="15" customHeight="1" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="A28" s="150">
+      <c r="A28" s="156">
         <f>A26 -1</f>
         <v>5</v>
       </c>
-      <c r="B28" s="140" t="s">
+      <c r="B28" s="154" t="s">
         <v>12</v>
       </c>
       <c r="C28" s="12">
@@ -2862,30 +2857,30 @@
       </c>
     </row>
     <row r="29" spans="1:17" ht="55.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A29" s="151"/>
-      <c r="B29" s="141"/>
+      <c r="A29" s="157"/>
+      <c r="B29" s="145"/>
       <c r="C29" s="15"/>
       <c r="D29" s="9" t="s">
-        <v>65</v>
+        <v>43</v>
       </c>
       <c r="E29" s="39" t="s">
-        <v>71</v>
+        <v>67</v>
       </c>
       <c r="F29" s="38" t="s">
-        <v>46</v>
+        <v>80</v>
       </c>
       <c r="G29" s="24"/>
       <c r="H29" s="11" t="s">
-        <v>45</v>
+        <v>62</v>
       </c>
       <c r="I29" s="25"/>
     </row>
     <row r="30" spans="1:17" ht="15.75" customHeight="1" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="A30" s="152">
+      <c r="A30" s="153">
         <f>A28 -1</f>
         <v>4</v>
       </c>
-      <c r="B30" s="141"/>
+      <c r="B30" s="145"/>
       <c r="C30" s="47">
         <f>I28 + 1</f>
         <v>13</v>
@@ -2916,21 +2911,21 @@
       </c>
     </row>
     <row r="31" spans="1:17" ht="92.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A31" s="146"/>
-      <c r="B31" s="141"/>
+      <c r="A31" s="139"/>
+      <c r="B31" s="145"/>
       <c r="C31" s="26"/>
       <c r="D31" s="72" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="E31" s="133" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="F31" s="23" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="G31" s="24"/>
       <c r="H31" s="55" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="I31" s="113" t="str">
         <f>H31</f>
@@ -2938,11 +2933,11 @@
       </c>
     </row>
     <row r="32" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A32" s="146">
+      <c r="A32" s="139">
         <f>A30 -1</f>
         <v>3</v>
       </c>
-      <c r="B32" s="141"/>
+      <c r="B32" s="145"/>
       <c r="C32" s="24">
         <f>I30 + 1</f>
         <v>20</v>
@@ -2973,8 +2968,8 @@
       </c>
     </row>
     <row r="33" spans="1:9" ht="52.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A33" s="146"/>
-      <c r="B33" s="141"/>
+      <c r="A33" s="139"/>
+      <c r="B33" s="145"/>
       <c r="C33" s="54" t="str">
         <f>I31</f>
         <v>Spring Break</v>
@@ -2985,21 +2980,21 @@
       </c>
       <c r="E33" s="10"/>
       <c r="F33" s="36" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="G33" s="115"/>
       <c r="H33" s="36" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="I33" s="116"/>
     </row>
     <row r="34" spans="1:9" ht="15" customHeight="1" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="A34" s="146">
+      <c r="A34" s="139">
         <f>A32 -1</f>
         <v>2</v>
       </c>
-      <c r="B34" s="141" t="s">
-        <v>29</v>
+      <c r="B34" s="145" t="s">
+        <v>28</v>
       </c>
       <c r="C34" s="26">
         <f>I32 + 1</f>
@@ -3031,11 +3026,11 @@
       </c>
     </row>
     <row r="35" spans="1:9" ht="58.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A35" s="147"/>
-      <c r="B35" s="145"/>
+      <c r="A35" s="140"/>
+      <c r="B35" s="146"/>
       <c r="C35" s="45"/>
       <c r="D35" s="35" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="E35" s="34"/>
       <c r="F35" s="114" t="s">
@@ -3048,11 +3043,11 @@
       <c r="I35" s="119"/>
     </row>
     <row r="36" spans="1:9" ht="15" customHeight="1" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="A36" s="153">
+      <c r="A36" s="141">
         <f>A34 -1</f>
         <v>1</v>
       </c>
-      <c r="B36" s="137" t="s">
+      <c r="B36" s="147" t="s">
         <v>5</v>
       </c>
       <c r="C36" s="111">
@@ -3085,29 +3080,29 @@
       </c>
     </row>
     <row r="37" spans="1:9" ht="90" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A37" s="149"/>
-      <c r="B37" s="138"/>
+      <c r="A37" s="142"/>
+      <c r="B37" s="148"/>
       <c r="C37" s="73"/>
       <c r="D37" s="6" t="s">
         <v>6</v>
       </c>
       <c r="E37" s="118"/>
       <c r="F37" s="69" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="G37" s="6"/>
       <c r="H37" s="6" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="I37" s="126" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
     </row>
     <row r="38" spans="1:9" ht="15.75" customHeight="1" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="A38" s="154" t="s">
-        <v>24</v>
-      </c>
-      <c r="B38" s="138"/>
+      <c r="A38" s="143" t="s">
+        <v>23</v>
+      </c>
+      <c r="B38" s="148"/>
       <c r="C38" s="18">
         <f>I36 + 1</f>
         <v>11</v>
@@ -3138,18 +3133,18 @@
       </c>
     </row>
     <row r="39" spans="1:9" ht="103.9" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A39" s="155"/>
-      <c r="B39" s="139"/>
+      <c r="A39" s="144"/>
+      <c r="B39" s="149"/>
       <c r="C39" s="90"/>
       <c r="D39" s="20" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="E39" s="49"/>
       <c r="F39" s="20" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
       <c r="G39" s="82" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="H39" s="59"/>
       <c r="I39" s="60"/>
@@ -3157,17 +3152,6 @@
     <row r="40" spans="1:9" ht="15.75" thickTop="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <mergeCells count="22">
-    <mergeCell ref="A34:A35"/>
-    <mergeCell ref="A36:A37"/>
-    <mergeCell ref="A38:A39"/>
-    <mergeCell ref="B34:B35"/>
-    <mergeCell ref="B36:B39"/>
-    <mergeCell ref="A1:I1"/>
-    <mergeCell ref="A3:A4"/>
-    <mergeCell ref="A5:A6"/>
-    <mergeCell ref="A7:A8"/>
-    <mergeCell ref="A9:A10"/>
-    <mergeCell ref="B3:B4"/>
     <mergeCell ref="B13:B16"/>
     <mergeCell ref="B22:B25"/>
     <mergeCell ref="B28:B33"/>
@@ -3179,6 +3163,17 @@
     <mergeCell ref="A28:A29"/>
     <mergeCell ref="A30:A31"/>
     <mergeCell ref="A32:A33"/>
+    <mergeCell ref="A1:I1"/>
+    <mergeCell ref="A3:A4"/>
+    <mergeCell ref="A5:A6"/>
+    <mergeCell ref="A7:A8"/>
+    <mergeCell ref="A9:A10"/>
+    <mergeCell ref="B3:B4"/>
+    <mergeCell ref="A34:A35"/>
+    <mergeCell ref="A36:A37"/>
+    <mergeCell ref="A38:A39"/>
+    <mergeCell ref="B34:B35"/>
+    <mergeCell ref="B36:B39"/>
   </mergeCells>
   <printOptions horizontalCentered="1" verticalCentered="1"/>
   <pageMargins left="0.25" right="0.25" top="0.25" bottom="0.25" header="0" footer="0"/>

</xml_diff>